<commit_message>
France daily ratings for 2026-03-29
</commit_message>
<xml_diff>
--- a/output/daily_ratings/france_ratings_2026-03-29.xlsx
+++ b/output/daily_ratings/france_ratings_2026-03-29.xlsx
@@ -998,10 +998,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>76.67338598291946</v>
+        <v>75.71695608961932</v>
       </c>
       <c r="T8" t="n">
-        <v>76.67338598291946</v>
+        <v>75.71695608961932</v>
       </c>
     </row>
     <row r="9">
@@ -1072,10 +1072,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>73.86047280685412</v>
+        <v>72.81956676022145</v>
       </c>
       <c r="T9" t="n">
-        <v>73.86047280685412</v>
+        <v>72.81956676022145</v>
       </c>
     </row>
     <row r="10">
@@ -1146,10 +1146,10 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>62.57121115238971</v>
+        <v>61.19127103721623</v>
       </c>
       <c r="T10" t="n">
-        <v>62.57121115238971</v>
+        <v>61.19127103721623</v>
       </c>
     </row>
     <row r="11">
@@ -1220,10 +1220,10 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>64.67858588176543</v>
+        <v>63.36193350411707</v>
       </c>
       <c r="T11" t="n">
-        <v>64.67858588176543</v>
+        <v>63.36193350411707</v>
       </c>
     </row>
     <row r="12">
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>66.0499052991259</v>
+        <v>64.77443577431302</v>
       </c>
       <c r="T12" t="n">
-        <v>66.0499052991259</v>
+        <v>64.77443577431302</v>
       </c>
     </row>
     <row r="13">
@@ -1368,10 +1368,10 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>59.55671556298448</v>
+        <v>58.08624546139065</v>
       </c>
       <c r="T13" t="n">
-        <v>59.55671556298448</v>
+        <v>58.08624546139065</v>
       </c>
     </row>
     <row r="14">
@@ -1442,10 +1442,10 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>58.54171141140753</v>
+        <v>57.04075915804615</v>
       </c>
       <c r="T14" t="n">
-        <v>58.54171141140753</v>
+        <v>57.04075915804615</v>
       </c>
     </row>
     <row r="15">
@@ -1863,7 +1863,7 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R20" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
@@ -1931,7 +1931,7 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R21" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
@@ -1999,7 +1999,7 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R22" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
@@ -2067,7 +2067,7 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R23" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
@@ -2135,7 +2135,7 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
@@ -2203,7 +2203,7 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R25" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
@@ -2271,7 +2271,7 @@
         <v>-2.541280000000015</v>
       </c>
       <c r="R26" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
@@ -2339,7 +2339,7 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R27" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
@@ -2407,7 +2407,7 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R28" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
@@ -2475,7 +2475,7 @@
         <v>-5.848210000000009</v>
       </c>
       <c r="R29" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
@@ -2543,7 +2543,7 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R30" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr"/>
@@ -2611,7 +2611,7 @@
         <v>-5.848210000000009</v>
       </c>
       <c r="R31" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
@@ -2679,7 +2679,7 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R32" t="n">
-        <v>0</v>
+        <v>10.80370635488746</v>
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr"/>
@@ -2754,10 +2754,10 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>65.59787587861555</v>
+        <v>64.30883120794934</v>
       </c>
       <c r="T33" t="n">
-        <v>65.59787587861555</v>
+        <v>64.30883120794934</v>
       </c>
     </row>
     <row r="34">
@@ -2828,10 +2828,10 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>63.5894620370138</v>
+        <v>62.24010157804597</v>
       </c>
       <c r="T34" t="n">
-        <v>63.5894620370138</v>
+        <v>62.24010157804597</v>
       </c>
     </row>
     <row r="35">
@@ -2902,10 +2902,10 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>60.21619821489585</v>
+        <v>58.76553340203153</v>
       </c>
       <c r="T35" t="n">
-        <v>60.21619821489585</v>
+        <v>58.76553340203153</v>
       </c>
     </row>
     <row r="36">
@@ -2976,10 +2976,10 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>51.26150463461434</v>
+        <v>49.54191645988792</v>
       </c>
       <c r="T36" t="n">
-        <v>51.26150463461434</v>
+        <v>49.54191645988792</v>
       </c>
     </row>
     <row r="37">
@@ -3050,10 +3050,10 @@
         <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>49.25309079301257</v>
+        <v>47.47318682998456</v>
       </c>
       <c r="T37" t="n">
-        <v>49.25309079301257</v>
+        <v>47.47318682998456</v>
       </c>
     </row>
     <row r="38">
@@ -3124,10 +3124,10 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>46.62326687920219</v>
+        <v>44.76438521786806</v>
       </c>
       <c r="T38" t="n">
-        <v>46.62326687920219</v>
+        <v>44.76438521786806</v>
       </c>
     </row>
     <row r="39">
@@ -3270,10 +3270,10 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>48.43980490932168</v>
+        <v>46.63547670753705</v>
       </c>
       <c r="T40" t="n">
-        <v>48.43980490932168</v>
+        <v>46.63547670753705</v>
       </c>
     </row>
     <row r="41">
@@ -3344,10 +3344,10 @@
         <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>52.69641088027898</v>
+        <v>51.01991516964209</v>
       </c>
       <c r="T41" t="n">
-        <v>52.69641088027898</v>
+        <v>51.01991516964209</v>
       </c>
     </row>
     <row r="42">
@@ -3418,10 +3418,10 @@
         <v>0</v>
       </c>
       <c r="S42" t="n">
-        <v>48.97441819109973</v>
+        <v>47.18614525683967</v>
       </c>
       <c r="T42" t="n">
-        <v>48.97441819109973</v>
+        <v>47.18614525683967</v>
       </c>
     </row>
     <row r="43">
@@ -3492,10 +3492,10 @@
         <v>0</v>
       </c>
       <c r="S43" t="n">
-        <v>46.16906477962127</v>
+        <v>44.29654272350545</v>
       </c>
       <c r="T43" t="n">
-        <v>46.16906477962127</v>
+        <v>44.29654272350545</v>
       </c>
     </row>
     <row r="44">
@@ -3566,10 +3566,10 @@
         <v>0</v>
       </c>
       <c r="S44" t="n">
-        <v>43.90118009603234</v>
+        <v>41.9605499390688</v>
       </c>
       <c r="T44" t="n">
-        <v>43.90118009603234</v>
+        <v>41.9605499390688</v>
       </c>
     </row>
     <row r="45">
@@ -3640,10 +3640,10 @@
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>48.25779322058037</v>
+        <v>46.44799892497626</v>
       </c>
       <c r="T45" t="n">
-        <v>48.25779322058037</v>
+        <v>46.44799892497626</v>
       </c>
     </row>
     <row r="46">
@@ -3714,10 +3714,10 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>40.25833649589222</v>
+        <v>38.20830608542981</v>
       </c>
       <c r="T46" t="n">
-        <v>40.25833649589222</v>
+        <v>38.20830608542981</v>
       </c>
     </row>
     <row r="47">
@@ -3788,10 +3788,10 @@
         <v>0</v>
       </c>
       <c r="S47" t="n">
-        <v>34.10587777587858</v>
+        <v>31.87107947047142</v>
       </c>
       <c r="T47" t="n">
-        <v>34.10587777587858</v>
+        <v>31.87107947047142</v>
       </c>
     </row>
     <row r="48">
@@ -3931,13 +3931,13 @@
         <v>-5.848210000000009</v>
       </c>
       <c r="R49" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S49" t="n">
-        <v>55.4755367173064</v>
+        <v>62.16795569996496</v>
       </c>
       <c r="T49" t="n">
-        <v>55.4755367173064</v>
+        <v>62.16795569996496</v>
       </c>
     </row>
     <row r="50">
@@ -4005,13 +4005,13 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R50" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S50" t="n">
-        <v>54.24391187481324</v>
+        <v>60.8993432497746</v>
       </c>
       <c r="T50" t="n">
-        <v>54.24391187481324</v>
+        <v>60.8993432497746</v>
       </c>
     </row>
     <row r="51">
@@ -4079,13 +4079,13 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R51" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S51" t="n">
-        <v>53.40874265670244</v>
+        <v>60.03909260237261</v>
       </c>
       <c r="T51" t="n">
-        <v>53.40874265670244</v>
+        <v>60.03909260237261</v>
       </c>
     </row>
     <row r="52">
@@ -4153,13 +4153,13 @@
         <v>-2.541280000000015</v>
       </c>
       <c r="R52" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S52" t="n">
-        <v>45.9913335998008</v>
+        <v>52.39892722645178</v>
       </c>
       <c r="T52" t="n">
-        <v>45.9913335998008</v>
+        <v>52.39892722645178</v>
       </c>
     </row>
     <row r="53">
@@ -4227,13 +4227,13 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R53" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S53" t="n">
-        <v>46.56035506819386</v>
+        <v>52.98503729367629</v>
       </c>
       <c r="T53" t="n">
-        <v>46.56035506819386</v>
+        <v>52.98503729367629</v>
       </c>
     </row>
     <row r="54">
@@ -4301,13 +4301,13 @@
         <v>2.970269999999999</v>
       </c>
       <c r="R54" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S54" t="n">
-        <v>49.33754247263257</v>
+        <v>55.8456279510155</v>
       </c>
       <c r="T54" t="n">
-        <v>49.33754247263257</v>
+        <v>55.8456279510155</v>
       </c>
     </row>
     <row r="55">
@@ -4375,13 +4375,13 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R55" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S55" t="n">
-        <v>46.14277045913845</v>
+        <v>52.55491196997528</v>
       </c>
       <c r="T55" t="n">
-        <v>46.14277045913845</v>
+        <v>52.55491196997528</v>
       </c>
     </row>
     <row r="56">
@@ -4449,13 +4449,13 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R56" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S56" t="n">
-        <v>44.47243202291685</v>
+        <v>50.8344106751713</v>
       </c>
       <c r="T56" t="n">
-        <v>44.47243202291685</v>
+        <v>50.8344106751713</v>
       </c>
     </row>
     <row r="57">
@@ -4523,7 +4523,7 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R57" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S57" t="inlineStr"/>
       <c r="T57" t="inlineStr"/>
@@ -4598,10 +4598,10 @@
         <v>0</v>
       </c>
       <c r="S58" t="n">
-        <v>69.89743269921769</v>
+        <v>68.73751040045033</v>
       </c>
       <c r="T58" t="n">
-        <v>69.89743269921769</v>
+        <v>68.73751040045033</v>
       </c>
     </row>
     <row r="59">
@@ -4672,10 +4672,10 @@
         <v>0</v>
       </c>
       <c r="S59" t="n">
-        <v>62.77099223240472</v>
+        <v>61.39705185348043</v>
       </c>
       <c r="T59" t="n">
-        <v>62.77099223240472</v>
+        <v>61.39705185348043</v>
       </c>
     </row>
     <row r="60">
@@ -4746,10 +4746,10 @@
         <v>0</v>
       </c>
       <c r="S60" t="n">
-        <v>65.94932613380479</v>
+        <v>64.67083606037914</v>
       </c>
       <c r="T60" t="n">
-        <v>65.94932613380479</v>
+        <v>64.67083606037914</v>
       </c>
     </row>
     <row r="61">
@@ -4820,10 +4820,10 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>55.63612242759232</v>
+        <v>54.04791082239363</v>
       </c>
       <c r="T61" t="n">
-        <v>55.63612242759232</v>
+        <v>54.04791082239363</v>
       </c>
     </row>
     <row r="62">
@@ -4894,10 +4894,10 @@
         <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>51.45390320884022</v>
+        <v>49.74009306224335</v>
       </c>
       <c r="T62" t="n">
-        <v>51.45390320884022</v>
+        <v>49.74009306224335</v>
       </c>
     </row>
     <row r="63">
@@ -5035,7 +5035,7 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R64" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr"/>
@@ -5103,7 +5103,7 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R65" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S65" t="inlineStr"/>
       <c r="T65" t="inlineStr"/>
@@ -5171,7 +5171,7 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R66" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S66" t="inlineStr"/>
       <c r="T66" t="inlineStr"/>
@@ -5239,7 +5239,7 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R67" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S67" t="inlineStr"/>
       <c r="T67" t="inlineStr"/>
@@ -5307,7 +5307,7 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R68" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S68" t="inlineStr"/>
       <c r="T68" t="inlineStr"/>
@@ -5375,7 +5375,7 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R69" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S69" t="inlineStr"/>
       <c r="T69" t="inlineStr"/>
@@ -5443,7 +5443,7 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R70" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S70" t="inlineStr"/>
       <c r="T70" t="inlineStr"/>
@@ -5511,7 +5511,7 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R71" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S71" t="inlineStr"/>
       <c r="T71" t="inlineStr"/>
@@ -5579,7 +5579,7 @@
         <v>-1.438970000000012</v>
       </c>
       <c r="R72" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S72" t="inlineStr"/>
       <c r="T72" t="inlineStr"/>
@@ -5654,10 +5654,10 @@
         <v>0</v>
       </c>
       <c r="S73" t="n">
-        <v>87.258127178846</v>
+        <v>86.61957351004526</v>
       </c>
       <c r="T73" t="n">
-        <v>87.258127178846</v>
+        <v>86.61957351004526</v>
       </c>
     </row>
     <row r="74">
@@ -5728,10 +5728,10 @@
         <v>0</v>
       </c>
       <c r="S74" t="n">
-        <v>81.30686033444687</v>
+        <v>80.48958087533452</v>
       </c>
       <c r="T74" t="n">
-        <v>81.30686033444687</v>
+        <v>80.48958087533452</v>
       </c>
     </row>
     <row r="75">
@@ -5802,10 +5802,10 @@
         <v>0</v>
       </c>
       <c r="S75" t="n">
-        <v>78.048517344999</v>
+        <v>77.13338478315717</v>
       </c>
       <c r="T75" t="n">
-        <v>78.048517344999</v>
+        <v>77.13338478315717</v>
       </c>
     </row>
     <row r="76">
@@ -5876,10 +5876,10 @@
         <v>0</v>
       </c>
       <c r="S76" t="n">
-        <v>81.20836225154224</v>
+        <v>80.38812474195564</v>
       </c>
       <c r="T76" t="n">
-        <v>81.20836225154224</v>
+        <v>80.38812474195564</v>
       </c>
     </row>
     <row r="77">
@@ -5950,10 +5950,10 @@
         <v>0</v>
       </c>
       <c r="S77" t="n">
-        <v>72.98610512282005</v>
+        <v>71.91894045605864</v>
       </c>
       <c r="T77" t="n">
-        <v>72.98610512282005</v>
+        <v>71.91894045605864</v>
       </c>
     </row>
     <row r="78">
@@ -6024,10 +6024,10 @@
         <v>0</v>
       </c>
       <c r="S78" t="n">
-        <v>78.03999422402194</v>
+        <v>77.12460569961408</v>
       </c>
       <c r="T78" t="n">
-        <v>78.03999422402194</v>
+        <v>77.12460569961408</v>
       </c>
     </row>
     <row r="79">
@@ -6098,10 +6098,10 @@
         <v>0</v>
       </c>
       <c r="S79" t="n">
-        <v>78.99167319451951</v>
+        <v>78.10486506829787</v>
       </c>
       <c r="T79" t="n">
-        <v>78.99167319451951</v>
+        <v>78.10486506829787</v>
       </c>
     </row>
     <row r="80">
@@ -6172,10 +6172,10 @@
         <v>0</v>
       </c>
       <c r="S80" t="n">
-        <v>72.89692078625197</v>
+        <v>71.82707777529035</v>
       </c>
       <c r="T80" t="n">
-        <v>72.89692078625197</v>
+        <v>71.82707777529035</v>
       </c>
     </row>
     <row r="81">
@@ -6246,10 +6246,10 @@
         <v>0</v>
       </c>
       <c r="S81" t="n">
-        <v>74.47684323952356</v>
+        <v>73.45444775468957</v>
       </c>
       <c r="T81" t="n">
-        <v>74.47684323952356</v>
+        <v>73.45444775468957</v>
       </c>
     </row>
     <row r="82">
@@ -6320,10 +6320,10 @@
         <v>0</v>
       </c>
       <c r="S82" t="n">
-        <v>72.41374411806532</v>
+        <v>71.32939056100662</v>
       </c>
       <c r="T82" t="n">
-        <v>72.41374411806532</v>
+        <v>71.32939056100662</v>
       </c>
     </row>
     <row r="83">
@@ -6394,10 +6394,10 @@
         <v>0</v>
       </c>
       <c r="S83" t="n">
-        <v>59.18337599446452</v>
+        <v>57.70169392553954</v>
       </c>
       <c r="T83" t="n">
-        <v>59.18337599446452</v>
+        <v>57.70169392553954</v>
       </c>
     </row>
     <row r="84">
@@ -6607,13 +6607,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R86" t="n">
-        <v>0</v>
+        <v>9.063867016622922</v>
       </c>
       <c r="S86" t="n">
-        <v>25.0201871358634</v>
+        <v>28.74658826782138</v>
       </c>
       <c r="T86" t="n">
-        <v>25.0201871358634</v>
+        <v>28.74658826782138</v>
       </c>
     </row>
     <row r="87">
@@ -6681,13 +6681,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R87" t="n">
-        <v>0</v>
+        <v>9.063867016622922</v>
       </c>
       <c r="S87" t="n">
-        <v>23.28186561349267</v>
+        <v>26.9560622491603</v>
       </c>
       <c r="T87" t="n">
-        <v>23.28186561349267</v>
+        <v>26.9560622491603</v>
       </c>
     </row>
     <row r="88">
@@ -6755,13 +6755,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R88" t="n">
-        <v>0</v>
+        <v>9.063867016622922</v>
       </c>
       <c r="S88" t="n">
-        <v>22.41270485230731</v>
+        <v>26.06079923982975</v>
       </c>
       <c r="T88" t="n">
-        <v>22.41270485230731</v>
+        <v>26.06079923982975</v>
       </c>
     </row>
     <row r="89">
@@ -6829,13 +6829,13 @@
         <v>-2.541280000000015</v>
       </c>
       <c r="R89" t="n">
-        <v>0</v>
+        <v>9.063867016622922</v>
       </c>
       <c r="S89" t="n">
-        <v>19.29465145200938</v>
+        <v>22.84910585114404</v>
       </c>
       <c r="T89" t="n">
-        <v>19.29465145200938</v>
+        <v>22.84910585114404</v>
       </c>
     </row>
     <row r="90">
@@ -6903,13 +6903,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R90" t="n">
-        <v>0</v>
+        <v>9.063867016622922</v>
       </c>
       <c r="S90" t="n">
-        <v>20.79027143142797</v>
+        <v>24.38964162241274</v>
       </c>
       <c r="T90" t="n">
-        <v>20.79027143142797</v>
+        <v>24.38964162241274</v>
       </c>
     </row>
     <row r="91">
@@ -6977,13 +6977,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R91" t="n">
-        <v>0</v>
+        <v>9.063867016622922</v>
       </c>
       <c r="S91" t="n">
-        <v>20.73232738068228</v>
+        <v>24.32995742179071</v>
       </c>
       <c r="T91" t="n">
-        <v>20.73232738068228</v>
+        <v>24.32995742179071</v>
       </c>
     </row>
     <row r="92">
@@ -7051,13 +7051,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R92" t="n">
-        <v>0</v>
+        <v>9.063867016622922</v>
       </c>
       <c r="S92" t="n">
-        <v>20.55849522844521</v>
+        <v>24.15090481992459</v>
       </c>
       <c r="T92" t="n">
-        <v>20.55849522844521</v>
+        <v>24.15090481992459</v>
       </c>
     </row>
     <row r="93">
@@ -7125,13 +7125,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R93" t="n">
-        <v>0</v>
+        <v>9.063867016622922</v>
       </c>
       <c r="S93" t="n">
-        <v>20.52372879799779</v>
+        <v>24.11509429955137</v>
       </c>
       <c r="T93" t="n">
-        <v>20.52372879799779</v>
+        <v>24.11509429955137</v>
       </c>
     </row>
     <row r="94">
@@ -7199,13 +7199,13 @@
         <v>-2.541280000000015</v>
       </c>
       <c r="R94" t="n">
-        <v>0</v>
+        <v>9.063867016622922</v>
       </c>
       <c r="S94" t="n">
-        <v>11.78510247536785</v>
+        <v>15.11403345052815</v>
       </c>
       <c r="T94" t="n">
-        <v>11.78510247536785</v>
+        <v>15.11403345052815</v>
       </c>
     </row>
     <row r="95">
@@ -7278,10 +7278,10 @@
         <v>0</v>
       </c>
       <c r="S95" t="n">
-        <v>72.00081344401215</v>
+        <v>70.90405893720717</v>
       </c>
       <c r="T95" t="n">
-        <v>72.00081344401215</v>
+        <v>70.90405893720717</v>
       </c>
     </row>
     <row r="96">
@@ -7352,10 +7352,10 @@
         <v>0</v>
       </c>
       <c r="S96" t="n">
-        <v>70.71913416758105</v>
+        <v>69.583888840654</v>
       </c>
       <c r="T96" t="n">
-        <v>70.71913416758105</v>
+        <v>69.583888840654</v>
       </c>
     </row>
     <row r="97">
@@ -7426,10 +7426,10 @@
         <v>0</v>
       </c>
       <c r="S97" t="n">
-        <v>68.38097976002695</v>
+        <v>67.17551602325764</v>
       </c>
       <c r="T97" t="n">
-        <v>68.38097976002695</v>
+        <v>67.17551602325764</v>
       </c>
     </row>
     <row r="98">
@@ -7500,10 +7500,10 @@
         <v>0</v>
       </c>
       <c r="S98" t="n">
-        <v>63.60945527111908</v>
+        <v>62.26069524003659</v>
       </c>
       <c r="T98" t="n">
-        <v>63.60945527111908</v>
+        <v>62.26069524003659</v>
       </c>
     </row>
     <row r="99">
@@ -7574,10 +7574,10 @@
         <v>0</v>
       </c>
       <c r="S99" t="n">
-        <v>59.7039745657349</v>
+        <v>58.23792688080211</v>
       </c>
       <c r="T99" t="n">
-        <v>59.7039745657349</v>
+        <v>58.23792688080211</v>
       </c>
     </row>
     <row r="100">
@@ -7648,10 +7648,10 @@
         <v>0</v>
       </c>
       <c r="S100" t="n">
-        <v>62.2930031969792</v>
+        <v>60.90470806463008</v>
       </c>
       <c r="T100" t="n">
-        <v>62.2930031969792</v>
+        <v>60.90470806463008</v>
       </c>
     </row>
     <row r="101">
@@ -7722,10 +7722,10 @@
         <v>0</v>
       </c>
       <c r="S101" t="n">
-        <v>58.48273816539466</v>
+        <v>56.98001485382392</v>
       </c>
       <c r="T101" t="n">
-        <v>58.48273816539466</v>
+        <v>56.98001485382392</v>
       </c>
     </row>
     <row r="102">
@@ -7796,10 +7796,10 @@
         <v>0</v>
       </c>
       <c r="S102" t="n">
-        <v>48.58449657076238</v>
+        <v>46.78451368439018</v>
       </c>
       <c r="T102" t="n">
-        <v>48.58449657076238</v>
+        <v>46.78451368439018</v>
       </c>
     </row>
     <row r="103">
@@ -7870,10 +7870,10 @@
         <v>0</v>
       </c>
       <c r="S103" t="n">
-        <v>46.85240900371505</v>
+        <v>45.00040883641707</v>
       </c>
       <c r="T103" t="n">
-        <v>46.85240900371505</v>
+        <v>45.00040883641707</v>
       </c>
     </row>
     <row r="104">
@@ -7944,10 +7944,10 @@
         <v>0</v>
       </c>
       <c r="S104" t="n">
-        <v>46.49721638689847</v>
+        <v>44.63454923342542</v>
       </c>
       <c r="T104" t="n">
-        <v>46.49721638689847</v>
+        <v>44.63454923342542</v>
       </c>
     </row>
     <row r="105">
@@ -8018,10 +8018,10 @@
         <v>0</v>
       </c>
       <c r="S105" t="n">
-        <v>45.69707711106171</v>
+        <v>43.81038053189286</v>
       </c>
       <c r="T105" t="n">
-        <v>45.69707711106171</v>
+        <v>43.81038053189286</v>
       </c>
     </row>
     <row r="106">
@@ -8092,10 +8092,10 @@
         <v>0</v>
       </c>
       <c r="S106" t="n">
-        <v>40.96032541986263</v>
+        <v>38.93137682752516</v>
       </c>
       <c r="T106" t="n">
-        <v>40.96032541986263</v>
+        <v>38.93137682752516</v>
       </c>
     </row>
     <row r="107">
@@ -8166,10 +8166,10 @@
         <v>0</v>
       </c>
       <c r="S107" t="n">
-        <v>48.86468196056535</v>
+        <v>47.0731134767961</v>
       </c>
       <c r="T107" t="n">
-        <v>48.86468196056535</v>
+        <v>47.0731134767961</v>
       </c>
     </row>
     <row r="108">
@@ -8452,10 +8452,10 @@
         <v>0</v>
       </c>
       <c r="S111" t="n">
-        <v>70.51930312406256</v>
+        <v>69.37805656040467</v>
       </c>
       <c r="T111" t="n">
-        <v>70.51930312406256</v>
+        <v>69.37805656040467</v>
       </c>
     </row>
     <row r="112">
@@ -8526,10 +8526,10 @@
         <v>0</v>
       </c>
       <c r="S112" t="n">
-        <v>57.6644978904372</v>
+        <v>56.13720155204206</v>
       </c>
       <c r="T112" t="n">
-        <v>57.6644978904372</v>
+        <v>56.13720155204206</v>
       </c>
     </row>
     <row r="113">
@@ -8600,10 +8600,10 @@
         <v>0</v>
       </c>
       <c r="S113" t="n">
-        <v>61.76207590435195</v>
+        <v>60.35783620045971</v>
       </c>
       <c r="T113" t="n">
-        <v>61.76207590435195</v>
+        <v>60.35783620045971</v>
       </c>
     </row>
     <row r="114">
@@ -8674,10 +8674,10 @@
         <v>0</v>
       </c>
       <c r="S114" t="n">
-        <v>55.72886367018783</v>
+        <v>54.14343722860401</v>
       </c>
       <c r="T114" t="n">
-        <v>55.72886367018783</v>
+        <v>54.14343722860401</v>
       </c>
     </row>
     <row r="115">
@@ -8748,10 +8748,10 @@
         <v>0</v>
       </c>
       <c r="S115" t="n">
-        <v>56.22160164849851</v>
+        <v>54.65097289401101</v>
       </c>
       <c r="T115" t="n">
-        <v>56.22160164849851</v>
+        <v>54.65097289401101</v>
       </c>
     </row>
     <row r="116">
@@ -8822,10 +8822,10 @@
         <v>0</v>
       </c>
       <c r="S116" t="n">
-        <v>59.36291808788365</v>
+        <v>57.88662794699341</v>
       </c>
       <c r="T116" t="n">
-        <v>59.36291808788365</v>
+        <v>57.88662794699341</v>
       </c>
     </row>
     <row r="117">
@@ -8896,10 +8896,10 @@
         <v>0</v>
       </c>
       <c r="S117" t="n">
-        <v>56.93454588932361</v>
+        <v>55.38532795814837</v>
       </c>
       <c r="T117" t="n">
-        <v>56.93454588932361</v>
+        <v>55.38532795814837</v>
       </c>
     </row>
     <row r="118">
@@ -8970,10 +8970,10 @@
         <v>0</v>
       </c>
       <c r="S118" t="n">
-        <v>48.77418668552091</v>
+        <v>46.9799004880321</v>
       </c>
       <c r="T118" t="n">
-        <v>48.77418668552091</v>
+        <v>46.9799004880321</v>
       </c>
     </row>
     <row r="119">
@@ -9044,10 +9044,10 @@
         <v>0</v>
       </c>
       <c r="S119" t="n">
-        <v>51.0809002172287</v>
+        <v>49.3558882112282</v>
       </c>
       <c r="T119" t="n">
-        <v>51.0809002172287</v>
+        <v>49.3558882112282</v>
       </c>
     </row>
     <row r="120">
@@ -9118,10 +9118,10 @@
         <v>0</v>
       </c>
       <c r="S120" t="n">
-        <v>51.13322567051057</v>
+        <v>49.4097850791745</v>
       </c>
       <c r="T120" t="n">
-        <v>51.13322567051057</v>
+        <v>49.4097850791745</v>
       </c>
     </row>
     <row r="121">
@@ -9192,10 +9192,10 @@
         <v>0</v>
       </c>
       <c r="S121" t="n">
-        <v>41.02554649362181</v>
+        <v>38.99855659146869</v>
       </c>
       <c r="T121" t="n">
-        <v>41.02554649362181</v>
+        <v>38.99855659146869</v>
       </c>
     </row>
     <row r="122">
@@ -9266,10 +9266,10 @@
         <v>0</v>
       </c>
       <c r="S122" t="n">
-        <v>51.0115670036583</v>
+        <v>49.28447281352555</v>
       </c>
       <c r="T122" t="n">
-        <v>51.0115670036583</v>
+        <v>49.28447281352555</v>
       </c>
     </row>
     <row r="123">
@@ -9340,10 +9340,10 @@
         <v>0</v>
       </c>
       <c r="S123" t="n">
-        <v>47.92257601755504</v>
+        <v>46.10271462848945</v>
       </c>
       <c r="T123" t="n">
-        <v>47.92257601755504</v>
+        <v>46.10271462848945</v>
       </c>
     </row>
     <row r="124">
@@ -9414,10 +9414,10 @@
         <v>0</v>
       </c>
       <c r="S124" t="n">
-        <v>37.3975953868276</v>
+        <v>35.26165247589049</v>
       </c>
       <c r="T124" t="n">
-        <v>37.3975953868276</v>
+        <v>35.26165247589049</v>
       </c>
     </row>
     <row r="125">
@@ -9488,10 +9488,10 @@
         <v>0</v>
       </c>
       <c r="S125" t="n">
-        <v>45.45595335601379</v>
+        <v>43.56201545582699</v>
       </c>
       <c r="T125" t="n">
-        <v>45.45595335601379</v>
+        <v>43.56201545582699</v>
       </c>
     </row>
     <row r="126">
@@ -9562,10 +9562,10 @@
         <v>0</v>
       </c>
       <c r="S126" t="n">
-        <v>45.87325480985247</v>
+        <v>43.99184912072013</v>
       </c>
       <c r="T126" t="n">
-        <v>45.87325480985247</v>
+        <v>43.99184912072013</v>
       </c>
     </row>
     <row r="127">
@@ -9638,10 +9638,10 @@
         <v>0</v>
       </c>
       <c r="S127" t="n">
-        <v>71.2653724379573</v>
+        <v>70.14653149502513</v>
       </c>
       <c r="T127" t="n">
-        <v>71.2653724379573</v>
+        <v>70.14653149502513</v>
       </c>
     </row>
     <row r="128">
@@ -9712,10 +9712,10 @@
         <v>0</v>
       </c>
       <c r="S128" t="n">
-        <v>69.3755072823449</v>
+        <v>68.19991075235026</v>
       </c>
       <c r="T128" t="n">
-        <v>69.3755072823449</v>
+        <v>68.19991075235026</v>
       </c>
     </row>
     <row r="129">
@@ -9786,10 +9786,10 @@
         <v>0</v>
       </c>
       <c r="S129" t="n">
-        <v>67.70448915601699</v>
+        <v>66.47870935528999</v>
       </c>
       <c r="T129" t="n">
-        <v>67.70448915601699</v>
+        <v>66.47870935528999</v>
       </c>
     </row>
     <row r="130">
@@ -9860,10 +9860,10 @@
         <v>0</v>
       </c>
       <c r="S130" t="n">
-        <v>69.49490056048069</v>
+        <v>68.32288959613965</v>
       </c>
       <c r="T130" t="n">
-        <v>69.49490056048069</v>
+        <v>68.32288959613965</v>
       </c>
     </row>
     <row r="131">
@@ -9934,10 +9934,10 @@
         <v>0</v>
       </c>
       <c r="S131" t="n">
-        <v>69.81320134091391</v>
+        <v>68.65074944357949</v>
       </c>
       <c r="T131" t="n">
-        <v>69.81320134091391</v>
+        <v>68.65074944357949</v>
       </c>
     </row>
     <row r="132">
@@ -10008,10 +10008,10 @@
         <v>0</v>
       </c>
       <c r="S132" t="n">
-        <v>68.24163696573473</v>
+        <v>67.03198854834443</v>
       </c>
       <c r="T132" t="n">
-        <v>68.24163696573473</v>
+        <v>67.03198854834443</v>
       </c>
     </row>
     <row r="133">
@@ -10082,10 +10082,10 @@
         <v>0</v>
       </c>
       <c r="S133" t="n">
-        <v>65.61571649810713</v>
+        <v>64.32720760896467</v>
       </c>
       <c r="T133" t="n">
-        <v>65.61571649810713</v>
+        <v>64.32720760896467</v>
       </c>
     </row>
     <row r="134">
@@ -10156,10 +10156,10 @@
         <v>0</v>
       </c>
       <c r="S134" t="n">
-        <v>65.19796196652516</v>
+        <v>63.89690725969961</v>
       </c>
       <c r="T134" t="n">
-        <v>65.19796196652516</v>
+        <v>63.89690725969961</v>
       </c>
     </row>
     <row r="135">
@@ -10230,10 +10230,10 @@
         <v>0</v>
       </c>
       <c r="S135" t="n">
-        <v>64.3624529033612</v>
+        <v>63.03630656116949</v>
       </c>
       <c r="T135" t="n">
-        <v>64.3624529033612</v>
+        <v>63.03630656116949</v>
       </c>
     </row>
     <row r="136">
@@ -10304,10 +10304,10 @@
         <v>0</v>
       </c>
       <c r="S136" t="n">
-        <v>66.15286430782487</v>
+        <v>64.88048680201911</v>
       </c>
       <c r="T136" t="n">
-        <v>66.15286430782487</v>
+        <v>64.88048680201911</v>
       </c>
     </row>
     <row r="137">
@@ -10378,10 +10378,10 @@
         <v>0</v>
       </c>
       <c r="S137" t="n">
-        <v>65.31735524466092</v>
+        <v>64.01988610348897</v>
       </c>
       <c r="T137" t="n">
-        <v>65.31735524466092</v>
+        <v>64.01988610348897</v>
       </c>
     </row>
     <row r="138">
@@ -10452,10 +10452,10 @@
         <v>0</v>
       </c>
       <c r="S138" t="n">
-        <v>61.97531899200511</v>
+        <v>60.57748330936847</v>
       </c>
       <c r="T138" t="n">
-        <v>61.97531899200511</v>
+        <v>60.57748330936847</v>
       </c>
     </row>
     <row r="139">
@@ -10526,10 +10526,10 @@
         <v>0</v>
       </c>
       <c r="S139" t="n">
-        <v>58.09613492963156</v>
+        <v>56.5818013221935</v>
       </c>
       <c r="T139" t="n">
-        <v>58.09613492963156</v>
+        <v>56.5818013221935</v>
       </c>
     </row>
     <row r="140">
@@ -10602,10 +10602,10 @@
         <v>0</v>
       </c>
       <c r="S140" t="n">
-        <v>53.13909804582999</v>
+        <v>51.47589691861418</v>
       </c>
       <c r="T140" t="n">
-        <v>53.13909804582999</v>
+        <v>51.47589691861418</v>
       </c>
     </row>
     <row r="141">
@@ -10676,10 +10676,10 @@
         <v>0</v>
       </c>
       <c r="S141" t="n">
-        <v>52.66307335623635</v>
+        <v>50.9855764679532</v>
       </c>
       <c r="T141" t="n">
-        <v>52.66307335623635</v>
+        <v>50.9855764679532</v>
       </c>
     </row>
     <row r="142">
@@ -10750,10 +10750,10 @@
         <v>0</v>
       </c>
       <c r="S142" t="n">
-        <v>49.97888273059705</v>
+        <v>48.22077542717751</v>
       </c>
       <c r="T142" t="n">
-        <v>49.97888273059705</v>
+        <v>48.22077542717751</v>
       </c>
     </row>
     <row r="143">
@@ -10824,10 +10824,10 @@
         <v>0</v>
       </c>
       <c r="S143" t="n">
-        <v>48.83880075137888</v>
+        <v>47.04645501468399</v>
       </c>
       <c r="T143" t="n">
-        <v>48.83880075137888</v>
+        <v>47.04645501468399</v>
       </c>
     </row>
     <row r="144">
@@ -10898,10 +10898,10 @@
         <v>0</v>
       </c>
       <c r="S144" t="n">
-        <v>47.95874939458228</v>
+        <v>46.13997434823439</v>
       </c>
       <c r="T144" t="n">
-        <v>47.95874939458228</v>
+        <v>46.13997434823439</v>
       </c>
     </row>
     <row r="145">
@@ -10972,10 +10972,10 @@
         <v>0</v>
       </c>
       <c r="S145" t="n">
-        <v>45.70210025847229</v>
+        <v>43.81555453222506</v>
       </c>
       <c r="T145" t="n">
-        <v>45.70210025847229</v>
+        <v>43.81555453222506</v>
       </c>
     </row>
     <row r="146">
@@ -11046,10 +11046,10 @@
         <v>0</v>
       </c>
       <c r="S146" t="n">
-        <v>38.21362618164704</v>
+        <v>36.10218994341273</v>
       </c>
       <c r="T146" t="n">
-        <v>38.21362618164704</v>
+        <v>36.10218994341273</v>
       </c>
     </row>
     <row r="147">
@@ -11122,10 +11122,10 @@
         <v>0</v>
       </c>
       <c r="S147" t="n">
-        <v>66.38992588630163</v>
+        <v>65.12466770803968</v>
       </c>
       <c r="T147" t="n">
-        <v>66.38992588630163</v>
+        <v>65.12466770803968</v>
       </c>
     </row>
     <row r="148">
@@ -11196,10 +11196,10 @@
         <v>0</v>
       </c>
       <c r="S148" t="n">
-        <v>67.66943488716043</v>
+        <v>66.44260235227296</v>
       </c>
       <c r="T148" t="n">
-        <v>67.66943488716043</v>
+        <v>66.44260235227296</v>
       </c>
     </row>
     <row r="149">
@@ -11270,10 +11270,10 @@
         <v>0</v>
       </c>
       <c r="S149" t="n">
-        <v>66.28217468115872</v>
+        <v>65.01368056678439</v>
       </c>
       <c r="T149" t="n">
-        <v>66.28217468115872</v>
+        <v>65.01368056678439</v>
       </c>
     </row>
     <row r="150">
@@ -11344,10 +11344,10 @@
         <v>0</v>
       </c>
       <c r="S150" t="n">
-        <v>63.79655670391272</v>
+        <v>62.45341561957195</v>
       </c>
       <c r="T150" t="n">
-        <v>63.79655670391272</v>
+        <v>62.45341561957195</v>
       </c>
     </row>
     <row r="151">
@@ -11418,10 +11418,10 @@
         <v>0</v>
       </c>
       <c r="S151" t="n">
-        <v>57.30740855116188</v>
+        <v>55.76938826506913</v>
       </c>
       <c r="T151" t="n">
-        <v>57.30740855116188</v>
+        <v>55.76938826506913</v>
       </c>
     </row>
     <row r="152">
@@ -11492,10 +11492,10 @@
         <v>0</v>
       </c>
       <c r="S152" t="n">
-        <v>52.69847505589895</v>
+        <v>51.0220413356632</v>
       </c>
       <c r="T152" t="n">
-        <v>52.69847505589895</v>
+        <v>51.0220413356632</v>
       </c>
     </row>
     <row r="153">
@@ -11566,10 +11566,10 @@
         <v>0</v>
       </c>
       <c r="S153" t="n">
-        <v>51.20346364475431</v>
+        <v>49.48213240891933</v>
       </c>
       <c r="T153" t="n">
-        <v>51.20346364475431</v>
+        <v>49.48213240891933</v>
       </c>
     </row>
     <row r="154">
@@ -11712,10 +11712,10 @@
         <v>0</v>
       </c>
       <c r="S155" t="n">
-        <v>63.70188639660388</v>
+        <v>62.35590221583757</v>
       </c>
       <c r="T155" t="n">
-        <v>63.70188639660388</v>
+        <v>62.35590221583757</v>
       </c>
     </row>
     <row r="156">
@@ -11786,10 +11786,10 @@
         <v>0</v>
       </c>
       <c r="S156" t="n">
-        <v>65.82810591269083</v>
+        <v>64.54597540767529</v>
       </c>
       <c r="T156" t="n">
-        <v>65.82810591269083</v>
+        <v>64.54597540767529</v>
       </c>
     </row>
     <row r="157">
@@ -11860,10 +11860,10 @@
         <v>0</v>
       </c>
       <c r="S157" t="n">
-        <v>64.7812391918778</v>
+        <v>63.46766965263304</v>
       </c>
       <c r="T157" t="n">
-        <v>64.7812391918778</v>
+        <v>63.46766965263304</v>
       </c>
     </row>
     <row r="158">
@@ -11934,10 +11934,10 @@
         <v>0</v>
       </c>
       <c r="S158" t="n">
-        <v>54.08370699490825</v>
+        <v>52.44887394215012</v>
       </c>
       <c r="T158" t="n">
-        <v>54.08370699490825</v>
+        <v>52.44887394215012</v>
       </c>
     </row>
     <row r="159">
@@ -12008,10 +12008,10 @@
         <v>0</v>
       </c>
       <c r="S159" t="n">
-        <v>53.56027363450172</v>
+        <v>51.90972106462898</v>
       </c>
       <c r="T159" t="n">
-        <v>53.56027363450172</v>
+        <v>51.90972106462898</v>
       </c>
     </row>
     <row r="160">
@@ -12082,10 +12082,10 @@
         <v>0</v>
       </c>
       <c r="S160" t="n">
-        <v>53.5927597089626</v>
+        <v>51.94318274638221</v>
       </c>
       <c r="T160" t="n">
-        <v>53.5927597089626</v>
+        <v>51.94318274638221</v>
       </c>
     </row>
     <row r="161">
@@ -12156,10 +12156,10 @@
         <v>0</v>
       </c>
       <c r="S161" t="n">
-        <v>42.04473970555826</v>
+        <v>40.04835775916418</v>
       </c>
       <c r="T161" t="n">
-        <v>42.04473970555826</v>
+        <v>40.04835775916418</v>
       </c>
     </row>
     <row r="162">
@@ -12232,10 +12232,10 @@
         <v>0</v>
       </c>
       <c r="S162" t="n">
-        <v>49.55913569190314</v>
+        <v>47.78842273271603</v>
       </c>
       <c r="T162" t="n">
-        <v>49.55913569190314</v>
+        <v>47.78842273271603</v>
       </c>
     </row>
     <row r="163">
@@ -12306,10 +12306,10 @@
         <v>0</v>
       </c>
       <c r="S163" t="n">
-        <v>42.67614894489898</v>
+        <v>40.69872919903493</v>
       </c>
       <c r="T163" t="n">
-        <v>42.67614894489898</v>
+        <v>40.69872919903493</v>
       </c>
     </row>
     <row r="164">
@@ -12380,10 +12380,10 @@
         <v>0</v>
       </c>
       <c r="S164" t="n">
-        <v>34.32105157386439</v>
+        <v>32.09271527194403</v>
       </c>
       <c r="T164" t="n">
-        <v>34.32105157386439</v>
+        <v>32.09271527194403</v>
       </c>
     </row>
     <row r="165">
@@ -12454,10 +12454,10 @@
         <v>0</v>
       </c>
       <c r="S165" t="n">
-        <v>36.81436647834411</v>
+        <v>34.66090829707436</v>
       </c>
       <c r="T165" t="n">
-        <v>36.81436647834411</v>
+        <v>34.66090829707436</v>
       </c>
     </row>
     <row r="166">
@@ -12528,10 +12528,10 @@
         <v>0</v>
       </c>
       <c r="S166" t="n">
-        <v>35.58103904088767</v>
+        <v>33.39054212034851</v>
       </c>
       <c r="T166" t="n">
-        <v>35.58103904088767</v>
+        <v>33.39054212034851</v>
       </c>
     </row>
     <row r="167">
@@ -12602,10 +12602,10 @@
         <v>0</v>
       </c>
       <c r="S167" t="n">
-        <v>34.67922635372538</v>
+        <v>32.46164659696996</v>
       </c>
       <c r="T167" t="n">
-        <v>34.67922635372538</v>
+        <v>32.46164659696996</v>
       </c>
     </row>
     <row r="168">
@@ -12676,10 +12676,10 @@
         <v>0</v>
       </c>
       <c r="S168" t="n">
-        <v>30.50167766820809</v>
+        <v>28.15863963342451</v>
       </c>
       <c r="T168" t="n">
-        <v>30.50167766820809</v>
+        <v>28.15863963342451</v>
       </c>
     </row>
     <row r="169">
@@ -12750,10 +12750,10 @@
         <v>0</v>
       </c>
       <c r="S169" t="n">
-        <v>29.5998649810458</v>
+        <v>27.22974411004597</v>
       </c>
       <c r="T169" t="n">
-        <v>29.5998649810458</v>
+        <v>27.22974411004597</v>
       </c>
     </row>
     <row r="170">
@@ -12824,10 +12824,10 @@
         <v>0</v>
       </c>
       <c r="S170" t="n">
-        <v>20.58173810942291</v>
+        <v>17.94078887626047</v>
       </c>
       <c r="T170" t="n">
-        <v>20.58173810942291</v>
+        <v>17.94078887626047</v>
       </c>
     </row>
     <row r="171">
@@ -13180,10 +13180,10 @@
         <v>0</v>
       </c>
       <c r="S175" t="n">
-        <v>66.90371104828034</v>
+        <v>65.65388263674299</v>
       </c>
       <c r="T175" t="n">
-        <v>66.90371104828034</v>
+        <v>65.65388263674299</v>
       </c>
     </row>
     <row r="176">
@@ -13254,10 +13254,10 @@
         <v>0</v>
       </c>
       <c r="S176" t="n">
-        <v>62.04020917696303</v>
+        <v>60.6443222474059</v>
       </c>
       <c r="T176" t="n">
-        <v>62.04020917696303</v>
+        <v>60.6443222474059</v>
       </c>
     </row>
     <row r="177">
@@ -13328,10 +13328,10 @@
         <v>0</v>
       </c>
       <c r="S177" t="n">
-        <v>54.51355169630472</v>
+        <v>52.89162754781469</v>
       </c>
       <c r="T177" t="n">
-        <v>54.51355169630472</v>
+        <v>52.89162754781469</v>
       </c>
     </row>
     <row r="178">
@@ -13402,10 +13402,10 @@
         <v>0</v>
       </c>
       <c r="S178" t="n">
-        <v>40.63141733428367</v>
+        <v>38.59259112108464</v>
       </c>
       <c r="T178" t="n">
-        <v>40.63141733428367</v>
+        <v>38.59259112108464</v>
       </c>
     </row>
     <row r="179">
@@ -13476,10 +13476,10 @@
         <v>0</v>
       </c>
       <c r="S179" t="n">
-        <v>30.47710797843804</v>
+        <v>28.13333207769472</v>
       </c>
       <c r="T179" t="n">
-        <v>30.47710797843804</v>
+        <v>28.13333207769472</v>
       </c>
     </row>
     <row r="180">
@@ -13550,10 +13550,10 @@
         <v>0</v>
       </c>
       <c r="S180" t="n">
-        <v>33.10475985362534</v>
+        <v>30.83989642149341</v>
       </c>
       <c r="T180" t="n">
-        <v>33.10475985362534</v>
+        <v>30.83989642149341</v>
       </c>
     </row>
     <row r="181">
@@ -13624,10 +13624,10 @@
         <v>0</v>
       </c>
       <c r="S181" t="n">
-        <v>33.36596110633019</v>
+        <v>31.10894195366692</v>
       </c>
       <c r="T181" t="n">
-        <v>33.36596110633019</v>
+        <v>31.10894195366692</v>
       </c>
     </row>
     <row r="182">
@@ -13840,10 +13840,10 @@
         <v>0</v>
       </c>
       <c r="S184" t="n">
-        <v>60.60825584082639</v>
+        <v>59.16936512764104</v>
       </c>
       <c r="T184" t="n">
-        <v>60.60825584082639</v>
+        <v>59.16936512764104</v>
       </c>
     </row>
     <row r="185">
@@ -13914,10 +13914,10 @@
         <v>0</v>
       </c>
       <c r="S185" t="n">
-        <v>55.38272539011666</v>
+        <v>53.78690387815869</v>
       </c>
       <c r="T185" t="n">
-        <v>55.38272539011666</v>
+        <v>53.78690387815869</v>
       </c>
     </row>
     <row r="186">
@@ -13988,10 +13988,10 @@
         <v>0</v>
       </c>
       <c r="S186" t="n">
-        <v>48.6850843153765</v>
+        <v>46.88812223526654</v>
       </c>
       <c r="T186" t="n">
-        <v>48.6850843153765</v>
+        <v>46.88812223526654</v>
       </c>
     </row>
     <row r="187">
@@ -14062,10 +14062,10 @@
         <v>0</v>
       </c>
       <c r="S187" t="n">
-        <v>46.80837440203685</v>
+        <v>44.95505180723027</v>
       </c>
       <c r="T187" t="n">
-        <v>46.80837440203685</v>
+        <v>44.95505180723027</v>
       </c>
     </row>
     <row r="188">
@@ -14136,10 +14136,10 @@
         <v>0</v>
       </c>
       <c r="S188" t="n">
-        <v>48.81424069342788</v>
+        <v>47.02115738003173</v>
       </c>
       <c r="T188" t="n">
-        <v>48.81424069342788</v>
+        <v>47.02115738003173</v>
       </c>
     </row>
     <row r="189">
@@ -14210,10 +14210,10 @@
         <v>0</v>
       </c>
       <c r="S189" t="n">
-        <v>46.93753078008823</v>
+        <v>45.08808695199546</v>
       </c>
       <c r="T189" t="n">
-        <v>46.93753078008823</v>
+        <v>45.08808695199546</v>
       </c>
     </row>
     <row r="190">
@@ -14284,10 +14284,10 @@
         <v>0</v>
       </c>
       <c r="S190" t="n">
-        <v>30.04714156003138</v>
+        <v>27.690453099669</v>
       </c>
       <c r="T190" t="n">
-        <v>30.04714156003138</v>
+        <v>27.690453099669</v>
       </c>
     </row>
     <row r="191">
@@ -14358,10 +14358,10 @@
         <v>0</v>
       </c>
       <c r="S191" t="n">
-        <v>22.8157448179306</v>
+        <v>20.24188627738519</v>
       </c>
       <c r="T191" t="n">
-        <v>22.8157448179306</v>
+        <v>20.24188627738519</v>
       </c>
     </row>
     <row r="192">
@@ -14784,10 +14784,10 @@
         <v>0</v>
       </c>
       <c r="S197" t="n">
-        <v>60.2353829414904</v>
+        <v>58.7852942757746</v>
       </c>
       <c r="T197" t="n">
-        <v>60.2353829414904</v>
+        <v>58.7852942757746</v>
       </c>
     </row>
     <row r="198">
@@ -14858,10 +14858,10 @@
         <v>0</v>
       </c>
       <c r="S198" t="n">
-        <v>58.6694802893069</v>
+        <v>57.17236513387388</v>
       </c>
       <c r="T198" t="n">
-        <v>58.6694802893069</v>
+        <v>57.17236513387388</v>
       </c>
     </row>
     <row r="199">
@@ -14932,10 +14932,10 @@
         <v>0</v>
       </c>
       <c r="S199" t="n">
-        <v>45.53859634787764</v>
+        <v>43.64714034514573</v>
       </c>
       <c r="T199" t="n">
-        <v>45.53859634787764</v>
+        <v>43.64714034514573</v>
       </c>
     </row>
     <row r="200">
@@ -15006,10 +15006,10 @@
         <v>0</v>
       </c>
       <c r="S200" t="n">
-        <v>46.54174683114275</v>
+        <v>44.68041699610097</v>
       </c>
       <c r="T200" t="n">
-        <v>46.54174683114275</v>
+        <v>44.68041699610097</v>
       </c>
     </row>
     <row r="201">
@@ -15080,10 +15080,10 @@
         <v>0</v>
       </c>
       <c r="S201" t="n">
-        <v>43.72798598655076</v>
+        <v>41.7821545413735</v>
       </c>
       <c r="T201" t="n">
-        <v>43.72798598655076</v>
+        <v>41.7821545413735</v>
       </c>
     </row>
     <row r="202">
@@ -15154,10 +15154,10 @@
         <v>0</v>
       </c>
       <c r="S202" t="n">
-        <v>39.44211451792834</v>
+        <v>37.36757169323624</v>
       </c>
       <c r="T202" t="n">
-        <v>39.44211451792834</v>
+        <v>37.36757169323624</v>
       </c>
     </row>
     <row r="203">
@@ -15228,10 +15228,10 @@
         <v>0</v>
       </c>
       <c r="S203" t="n">
-        <v>38.50419423639767</v>
+        <v>36.40148420832708</v>
       </c>
       <c r="T203" t="n">
-        <v>38.50419423639767</v>
+        <v>36.40148420832708</v>
       </c>
     </row>
     <row r="204">
@@ -15302,10 +15302,10 @@
         <v>0</v>
       </c>
       <c r="S204" t="n">
-        <v>32.68098194201038</v>
+        <v>30.40339180073395</v>
       </c>
       <c r="T204" t="n">
-        <v>32.68098194201038</v>
+        <v>30.40339180073395</v>
       </c>
     </row>
     <row r="205">
@@ -15376,10 +15376,10 @@
         <v>0</v>
       </c>
       <c r="S205" t="n">
-        <v>29.33303075491863</v>
+        <v>26.95489643750584</v>
       </c>
       <c r="T205" t="n">
-        <v>29.33303075491863</v>
+        <v>26.95489643750584</v>
       </c>
     </row>
     <row r="206">
@@ -15450,10 +15450,10 @@
         <v>0</v>
       </c>
       <c r="S206" t="n">
-        <v>32.40771240644838</v>
+        <v>30.12191555641759</v>
       </c>
       <c r="T206" t="n">
-        <v>32.40771240644838</v>
+        <v>30.12191555641759</v>
       </c>
     </row>
     <row r="207">
@@ -15524,10 +15524,10 @@
         <v>0</v>
       </c>
       <c r="S207" t="n">
-        <v>31.06606218588683</v>
+        <v>28.73997349509994</v>
       </c>
       <c r="T207" t="n">
-        <v>31.06606218588683</v>
+        <v>28.73997349509994</v>
       </c>
     </row>
     <row r="208">
@@ -15880,10 +15880,10 @@
         <v>0</v>
       </c>
       <c r="S212" t="n">
-        <v>70.3256294664005</v>
+        <v>69.17856658187628</v>
       </c>
       <c r="T212" t="n">
-        <v>70.3256294664005</v>
+        <v>69.17856658187628</v>
       </c>
     </row>
     <row r="213">
@@ -15954,10 +15954,10 @@
         <v>0</v>
       </c>
       <c r="S213" t="n">
-        <v>58.49206527256383</v>
+        <v>56.98962206851367</v>
       </c>
       <c r="T213" t="n">
-        <v>58.49206527256383</v>
+        <v>56.98962206851367</v>
       </c>
     </row>
     <row r="214">
@@ -16028,10 +16028,10 @@
         <v>0</v>
       </c>
       <c r="S214" t="n">
-        <v>57.81777142513244</v>
+        <v>56.29507812913793</v>
       </c>
       <c r="T214" t="n">
-        <v>57.81777142513244</v>
+        <v>56.29507812913793</v>
       </c>
     </row>
     <row r="215">
@@ -16102,10 +16102,10 @@
         <v>0</v>
       </c>
       <c r="S215" t="n">
-        <v>49.84976818512333</v>
+        <v>48.0877833712873</v>
       </c>
       <c r="T215" t="n">
-        <v>49.84976818512333</v>
+        <v>48.0877833712873</v>
       </c>
     </row>
     <row r="216">
@@ -16176,10 +16176,10 @@
         <v>0</v>
       </c>
       <c r="S216" t="n">
-        <v>52.1196955857528</v>
+        <v>50.42588021873116</v>
       </c>
       <c r="T216" t="n">
-        <v>52.1196955857528</v>
+        <v>50.42588021873116</v>
       </c>
     </row>
     <row r="217">
@@ -16250,10 +16250,10 @@
         <v>0</v>
       </c>
       <c r="S217" t="n">
-        <v>45.68048217136731</v>
+        <v>43.79328722037451</v>
       </c>
       <c r="T217" t="n">
-        <v>45.68048217136731</v>
+        <v>43.79328722037451</v>
       </c>
     </row>
     <row r="218">
@@ -16324,10 +16324,10 @@
         <v>0</v>
       </c>
       <c r="S218" t="n">
-        <v>37.47371250840116</v>
+        <v>35.34005551289436</v>
       </c>
       <c r="T218" t="n">
-        <v>37.47371250840116</v>
+        <v>35.34005551289436</v>
       </c>
     </row>
     <row r="219">
@@ -16470,10 +16470,10 @@
         <v>0</v>
       </c>
       <c r="S220" t="n">
-        <v>83.57565950730648</v>
+        <v>82.82651561257558</v>
       </c>
       <c r="T220" t="n">
-        <v>83.57565950730648</v>
+        <v>82.82651561257558</v>
       </c>
     </row>
     <row r="221">
@@ -16544,10 +16544,10 @@
         <v>0</v>
       </c>
       <c r="S221" t="n">
-        <v>71.80330828049688</v>
+        <v>70.70062238675146</v>
       </c>
       <c r="T221" t="n">
-        <v>71.80330828049688</v>
+        <v>70.70062238675146</v>
       </c>
     </row>
     <row r="222">
@@ -16618,10 +16618,10 @@
         <v>0</v>
       </c>
       <c r="S222" t="n">
-        <v>64.23763508883621</v>
+        <v>62.90774027373457</v>
       </c>
       <c r="T222" t="n">
-        <v>64.23763508883621</v>
+        <v>62.90774027373457</v>
       </c>
     </row>
     <row r="223">
@@ -16692,10 +16692,10 @@
         <v>0</v>
       </c>
       <c r="S223" t="n">
-        <v>48.16057955655727</v>
+        <v>46.34786578357365</v>
       </c>
       <c r="T223" t="n">
-        <v>48.16057955655727</v>
+        <v>46.34786578357365</v>
       </c>
     </row>
     <row r="224">
@@ -16978,10 +16978,10 @@
         <v>0</v>
       </c>
       <c r="S227" t="n">
-        <v>55.50429135727116</v>
+        <v>53.91212066019392</v>
       </c>
       <c r="T227" t="n">
-        <v>55.50429135727116</v>
+        <v>53.91212066019392</v>
       </c>
     </row>
     <row r="228">
@@ -17052,10 +17052,10 @@
         <v>0</v>
       </c>
       <c r="S228" t="n">
-        <v>50.95486266964176</v>
+        <v>49.2260655602523</v>
       </c>
       <c r="T228" t="n">
-        <v>50.95486266964176</v>
+        <v>49.2260655602523</v>
       </c>
     </row>
     <row r="229">
@@ -17126,10 +17126,10 @@
         <v>0</v>
       </c>
       <c r="S229" t="n">
-        <v>47.4312066698787</v>
+        <v>45.5965886958213</v>
       </c>
       <c r="T229" t="n">
-        <v>47.4312066698787</v>
+        <v>45.5965886958213</v>
       </c>
     </row>
     <row r="230">
@@ -17200,10 +17200,10 @@
         <v>0</v>
       </c>
       <c r="S230" t="n">
-        <v>45.11346766306987</v>
+        <v>43.20924438537568</v>
       </c>
       <c r="T230" t="n">
-        <v>45.11346766306987</v>
+        <v>43.20924438537568</v>
       </c>
     </row>
     <row r="231">
@@ -17274,10 +17274,10 @@
         <v>0</v>
       </c>
       <c r="S231" t="n">
-        <v>38.51249359970783</v>
+        <v>36.41003281441285</v>
       </c>
       <c r="T231" t="n">
-        <v>38.51249359970783</v>
+        <v>36.41003281441285</v>
       </c>
     </row>
     <row r="232">
@@ -17348,10 +17348,10 @@
         <v>0</v>
       </c>
       <c r="S232" t="n">
-        <v>24.59801390574346</v>
+        <v>22.0776796751636</v>
       </c>
       <c r="T232" t="n">
-        <v>24.59801390574346</v>
+        <v>22.0776796751636</v>
       </c>
     </row>
     <row r="233">
@@ -17422,10 +17422,10 @@
         <v>0</v>
       </c>
       <c r="S233" t="n">
-        <v>12.1085973462597</v>
+        <v>9.213186530561574</v>
       </c>
       <c r="T233" t="n">
-        <v>12.1085973462597</v>
+        <v>9.213186530561574</v>
       </c>
     </row>
     <row r="234">
@@ -17638,10 +17638,10 @@
         <v>0</v>
       </c>
       <c r="S236" t="n">
-        <v>57.09818426111585</v>
+        <v>55.55388064450398</v>
       </c>
       <c r="T236" t="n">
-        <v>57.09818426111585</v>
+        <v>55.55388064450398</v>
       </c>
     </row>
     <row r="237">
@@ -17712,10 +17712,10 @@
         <v>0</v>
       </c>
       <c r="S237" t="n">
-        <v>61.07180668260186</v>
+        <v>59.64683712145221</v>
       </c>
       <c r="T237" t="n">
-        <v>61.07180668260186</v>
+        <v>59.64683712145221</v>
       </c>
     </row>
     <row r="238">
@@ -17786,10 +17786,10 @@
         <v>0</v>
       </c>
       <c r="S238" t="n">
-        <v>62.10120785602701</v>
+        <v>60.70715281158085</v>
       </c>
       <c r="T238" t="n">
-        <v>62.10120785602701</v>
+        <v>60.70715281158085</v>
       </c>
     </row>
     <row r="239">
@@ -17860,10 +17860,10 @@
         <v>0</v>
       </c>
       <c r="S239" t="n">
-        <v>42.05682557449752</v>
+        <v>40.06080658552649</v>
       </c>
       <c r="T239" t="n">
-        <v>42.05682557449752</v>
+        <v>40.06080658552649</v>
       </c>
     </row>
     <row r="240">
@@ -17934,10 +17934,10 @@
         <v>0</v>
       </c>
       <c r="S240" t="n">
-        <v>40.2752251381147</v>
+        <v>38.22570191981951</v>
       </c>
       <c r="T240" t="n">
-        <v>40.2752251381147</v>
+        <v>38.22570191981951</v>
       </c>
     </row>
     <row r="241">
@@ -18008,10 +18008,10 @@
         <v>0</v>
       </c>
       <c r="S241" t="n">
-        <v>30.11443304211623</v>
+        <v>27.75976544951719</v>
       </c>
       <c r="T241" t="n">
-        <v>30.11443304211623</v>
+        <v>27.75976544951719</v>
       </c>
     </row>
     <row r="242">
@@ -18082,10 +18082,10 @@
         <v>0</v>
       </c>
       <c r="S242" t="n">
-        <v>34.52000228024588</v>
+        <v>32.29764077716428</v>
       </c>
       <c r="T242" t="n">
-        <v>34.52000228024588</v>
+        <v>32.29764077716428</v>
       </c>
     </row>
     <row r="243">
@@ -18228,10 +18228,10 @@
         <v>0</v>
       </c>
       <c r="S244" t="n">
-        <v>50.46765956436265</v>
+        <v>48.72423098871399</v>
       </c>
       <c r="T244" t="n">
-        <v>50.46765956436265</v>
+        <v>48.72423098871399</v>
       </c>
     </row>
     <row r="245">
@@ -18302,10 +18302,10 @@
         <v>0</v>
       </c>
       <c r="S245" t="n">
-        <v>46.44678381774956</v>
+        <v>44.58260209586372</v>
       </c>
       <c r="T245" t="n">
-        <v>46.44678381774956</v>
+        <v>44.58260209586372</v>
       </c>
     </row>
     <row r="246">
@@ -18376,10 +18376,10 @@
         <v>0</v>
       </c>
       <c r="S246" t="n">
-        <v>49.25476539119563</v>
+        <v>47.47491171895302</v>
       </c>
       <c r="T246" t="n">
-        <v>49.25476539119563</v>
+        <v>47.47491171895302</v>
       </c>
     </row>
     <row r="247">
@@ -18450,10 +18450,10 @@
         <v>0</v>
       </c>
       <c r="S247" t="n">
-        <v>40.01338262316864</v>
+        <v>37.95599586730329</v>
       </c>
       <c r="T247" t="n">
-        <v>40.01338262316864</v>
+        <v>37.95599586730329</v>
       </c>
     </row>
     <row r="248">
@@ -18524,10 +18524,10 @@
         <v>0</v>
       </c>
       <c r="S248" t="n">
-        <v>31.56291210609807</v>
+        <v>29.25174459041183</v>
       </c>
       <c r="T248" t="n">
-        <v>31.56291210609807</v>
+        <v>29.25174459041183</v>
       </c>
     </row>
     <row r="249">
@@ -18670,10 +18670,10 @@
         <v>0</v>
       </c>
       <c r="S250" t="n">
-        <v>69.88353817232982</v>
+        <v>68.72319859933094</v>
       </c>
       <c r="T250" t="n">
-        <v>69.88353817232982</v>
+        <v>68.72319859933094</v>
       </c>
     </row>
     <row r="251">
@@ -18744,10 +18744,10 @@
         <v>0</v>
       </c>
       <c r="S251" t="n">
-        <v>58.89642067458443</v>
+        <v>57.4061208915373</v>
       </c>
       <c r="T251" t="n">
-        <v>58.89642067458443</v>
+        <v>57.4061208915373</v>
       </c>
     </row>
     <row r="252">
@@ -18818,10 +18818,10 @@
         <v>0</v>
       </c>
       <c r="S252" t="n">
-        <v>53.96833145534388</v>
+        <v>52.33003349586413</v>
       </c>
       <c r="T252" t="n">
-        <v>53.96833145534388</v>
+        <v>52.33003349586413</v>
       </c>
     </row>
     <row r="253">
@@ -18892,10 +18892,10 @@
         <v>0</v>
       </c>
       <c r="S253" t="n">
-        <v>47.39754582968979</v>
+        <v>45.56191696829989</v>
       </c>
       <c r="T253" t="n">
-        <v>47.39754582968979</v>
+        <v>45.56191696829989</v>
       </c>
     </row>
     <row r="254">
@@ -18966,10 +18966,10 @@
         <v>0</v>
       </c>
       <c r="S254" t="n">
-        <v>44.93350122006952</v>
+        <v>43.02387327046331</v>
       </c>
       <c r="T254" t="n">
-        <v>44.93350122006952</v>
+        <v>43.02387327046331</v>
       </c>
     </row>
     <row r="255">
@@ -19040,10 +19040,10 @@
         <v>0</v>
       </c>
       <c r="S255" t="n">
-        <v>48.11781078735068</v>
+        <v>46.30381260177442</v>
       </c>
       <c r="T255" t="n">
-        <v>48.11781078735068</v>
+        <v>46.30381260177442</v>
       </c>
     </row>
     <row r="256">
@@ -19114,10 +19114,10 @@
         <v>0</v>
       </c>
       <c r="S256" t="n">
-        <v>42.8801307120526</v>
+        <v>40.90883685559948</v>
       </c>
       <c r="T256" t="n">
-        <v>42.8801307120526</v>
+        <v>40.90883685559948</v>
       </c>
     </row>
     <row r="257">
@@ -19188,10 +19188,10 @@
         <v>0</v>
       </c>
       <c r="S257" t="n">
-        <v>37.44028414566278</v>
+        <v>35.30562324448253</v>
       </c>
       <c r="T257" t="n">
-        <v>37.44028414566278</v>
+        <v>35.30562324448253</v>
       </c>
     </row>
     <row r="258">
@@ -19331,13 +19331,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R259" t="n">
-        <v>0</v>
+        <v>12.54354569315199</v>
       </c>
       <c r="S259" t="n">
-        <v>59.52884589083887</v>
+        <v>66.68489144290291</v>
       </c>
       <c r="T259" t="n">
-        <v>59.52884589083887</v>
+        <v>66.68489144290291</v>
       </c>
     </row>
     <row r="260">
@@ -19405,13 +19405,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R260" t="n">
-        <v>0</v>
+        <v>12.54354569315199</v>
       </c>
       <c r="S260" t="n">
-        <v>45.97059949427648</v>
+        <v>52.71946984048569</v>
       </c>
       <c r="T260" t="n">
-        <v>45.97059949427648</v>
+        <v>52.71946984048569</v>
       </c>
     </row>
     <row r="261">
@@ -19479,13 +19479,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R261" t="n">
-        <v>0</v>
+        <v>12.54354569315199</v>
       </c>
       <c r="S261" t="n">
-        <v>36.28613778244621</v>
+        <v>42.74416869590197</v>
       </c>
       <c r="T261" t="n">
-        <v>36.28613778244621</v>
+        <v>42.74416869590197</v>
       </c>
     </row>
     <row r="262">
@@ -19553,13 +19553,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R262" t="n">
-        <v>0</v>
+        <v>12.54354569315199</v>
       </c>
       <c r="S262" t="n">
-        <v>32.4123530977141</v>
+        <v>38.75404823806847</v>
       </c>
       <c r="T262" t="n">
-        <v>32.4123530977141</v>
+        <v>38.75404823806847</v>
       </c>
     </row>
     <row r="263">
@@ -19627,7 +19627,7 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R263" t="n">
-        <v>0</v>
+        <v>12.54354569315199</v>
       </c>
       <c r="S263" t="inlineStr"/>
       <c r="T263" t="inlineStr"/>
@@ -19697,7 +19697,7 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R264" t="n">
-        <v>0</v>
+        <v>12.54354569315199</v>
       </c>
       <c r="S264" t="inlineStr"/>
       <c r="T264" t="inlineStr"/>
@@ -19772,10 +19772,10 @@
         <v>0</v>
       </c>
       <c r="S265" t="n">
-        <v>66.08099075226349</v>
+        <v>64.80645477190836</v>
       </c>
       <c r="T265" t="n">
-        <v>66.08099075226349</v>
+        <v>64.80645477190836</v>
       </c>
     </row>
     <row r="266">
@@ -19846,10 +19846,10 @@
         <v>0</v>
       </c>
       <c r="S266" t="n">
-        <v>64.26488442082146</v>
+        <v>62.93580794549886</v>
       </c>
       <c r="T266" t="n">
-        <v>64.26488442082146</v>
+        <v>62.93580794549886</v>
       </c>
     </row>
     <row r="267">
@@ -19920,10 +19920,10 @@
         <v>0</v>
       </c>
       <c r="S267" t="n">
-        <v>61.84340931223203</v>
+        <v>60.44161217695285</v>
       </c>
       <c r="T267" t="n">
-        <v>61.84340931223203</v>
+        <v>60.44161217695285</v>
       </c>
     </row>
     <row r="268">
@@ -19994,10 +19994,10 @@
         <v>0</v>
       </c>
       <c r="S268" t="n">
-        <v>57.00045909505321</v>
+        <v>55.45322063986082</v>
       </c>
       <c r="T268" t="n">
-        <v>57.00045909505321</v>
+        <v>55.45322063986082</v>
       </c>
     </row>
     <row r="269">
@@ -20068,10 +20068,10 @@
         <v>0</v>
       </c>
       <c r="S269" t="n">
-        <v>56.75831158419427</v>
+        <v>55.20380106300622</v>
       </c>
       <c r="T269" t="n">
-        <v>56.75831158419427</v>
+        <v>55.20380106300622</v>
       </c>
     </row>
     <row r="270">
@@ -20142,10 +20142,10 @@
         <v>0</v>
       </c>
       <c r="S270" t="n">
-        <v>47.07241114983663</v>
+        <v>45.22701798882217</v>
       </c>
       <c r="T270" t="n">
-        <v>47.07241114983663</v>
+        <v>45.22701798882217</v>
       </c>
     </row>
     <row r="271">
@@ -20216,10 +20216,10 @@
         <v>0</v>
       </c>
       <c r="S271" t="n">
-        <v>46.46704237268928</v>
+        <v>44.60346904668566</v>
       </c>
       <c r="T271" t="n">
-        <v>46.46704237268928</v>
+        <v>44.60346904668566</v>
       </c>
     </row>
     <row r="272">
@@ -20290,10 +20290,10 @@
         <v>0</v>
       </c>
       <c r="S272" t="n">
-        <v>45.25630481839457</v>
+        <v>43.35637116241265</v>
       </c>
       <c r="T272" t="n">
-        <v>45.25630481839457</v>
+        <v>43.35637116241265</v>
       </c>
     </row>
     <row r="273">
@@ -20364,10 +20364,10 @@
         <v>0</v>
       </c>
       <c r="S273" t="n">
-        <v>33.14892927544752</v>
+        <v>30.88539231968259</v>
       </c>
       <c r="T273" t="n">
-        <v>33.14892927544752</v>
+        <v>30.88539231968259</v>
       </c>
     </row>
     <row r="274">
@@ -20438,10 +20438,10 @@
         <v>0</v>
       </c>
       <c r="S274" t="n">
-        <v>31.93819172115281</v>
+        <v>29.63829443540958</v>
       </c>
       <c r="T274" t="n">
-        <v>31.93819172115281</v>
+        <v>29.63829443540958</v>
       </c>
     </row>
     <row r="275">
@@ -20512,10 +20512,10 @@
         <v>0</v>
       </c>
       <c r="S275" t="n">
-        <v>30.12208538971075</v>
+        <v>27.76764760900006</v>
       </c>
       <c r="T275" t="n">
-        <v>30.12208538971075</v>
+        <v>27.76764760900006</v>
       </c>
     </row>
     <row r="276">
@@ -20586,10 +20586,10 @@
         <v>0</v>
       </c>
       <c r="S276" t="n">
-        <v>29.5167166125634</v>
+        <v>27.14409866686356</v>
       </c>
       <c r="T276" t="n">
-        <v>29.5167166125634</v>
+        <v>27.14409866686356</v>
       </c>
     </row>
     <row r="277">
@@ -20659,13 +20659,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R277" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S277" t="n">
-        <v>59.04229671584907</v>
+        <v>66.49767614246426</v>
       </c>
       <c r="T277" t="n">
-        <v>59.04229671584907</v>
+        <v>66.49767614246426</v>
       </c>
     </row>
     <row r="278">
@@ -20733,13 +20733,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R278" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S278" t="n">
-        <v>55.9557385240998</v>
+        <v>63.31842381237663</v>
       </c>
       <c r="T278" t="n">
-        <v>55.9557385240998</v>
+        <v>63.31842381237663</v>
       </c>
     </row>
     <row r="279">
@@ -20807,13 +20807,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R279" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S279" t="n">
-        <v>31.26327299010561</v>
+        <v>37.8844051716756</v>
       </c>
       <c r="T279" t="n">
-        <v>31.26327299010561</v>
+        <v>37.8844051716756</v>
       </c>
     </row>
     <row r="280">
@@ -20881,13 +20881,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R280" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S280" t="n">
-        <v>30.74884662481406</v>
+        <v>37.35452978332766</v>
       </c>
       <c r="T280" t="n">
-        <v>30.74884662481406</v>
+        <v>37.35452978332766</v>
       </c>
     </row>
     <row r="281">
@@ -20955,13 +20955,13 @@
         <v>-4.745900000000006</v>
       </c>
       <c r="R281" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S281" t="n">
-        <v>20.46031931898314</v>
+        <v>26.7570220163689</v>
       </c>
       <c r="T281" t="n">
-        <v>20.46031931898314</v>
+        <v>26.7570220163689</v>
       </c>
     </row>
     <row r="282">
@@ -21031,13 +21031,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R282" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S282" t="n">
-        <v>52.24241572669569</v>
+        <v>58.83773906243938</v>
       </c>
       <c r="T282" t="n">
-        <v>52.24241572669569</v>
+        <v>58.83773906243938</v>
       </c>
     </row>
     <row r="283">
@@ -21105,13 +21105,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R283" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S283" t="n">
-        <v>42.13451994124446</v>
+        <v>48.4262874610794</v>
       </c>
       <c r="T283" t="n">
-        <v>42.13451994124446</v>
+        <v>48.4262874610794</v>
       </c>
     </row>
     <row r="284">
@@ -21179,13 +21179,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R284" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S284" t="n">
-        <v>41.90126080773404</v>
+        <v>48.1860231933557</v>
       </c>
       <c r="T284" t="n">
-        <v>41.90126080773404</v>
+        <v>48.1860231933557</v>
       </c>
     </row>
     <row r="285">
@@ -21253,13 +21253,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R285" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S285" t="n">
-        <v>41.66800167422363</v>
+        <v>47.94575892563201</v>
       </c>
       <c r="T285" t="n">
-        <v>41.66800167422363</v>
+        <v>47.94575892563201</v>
       </c>
     </row>
     <row r="286">
@@ -21327,13 +21327,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R286" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S286" t="n">
-        <v>41.59024862972016</v>
+        <v>47.86567083639078</v>
       </c>
       <c r="T286" t="n">
-        <v>41.59024862972016</v>
+        <v>47.86567083639078</v>
       </c>
     </row>
     <row r="287">
@@ -21401,13 +21401,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R287" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S287" t="n">
-        <v>41.20148340720281</v>
+        <v>47.46523039018463</v>
       </c>
       <c r="T287" t="n">
-        <v>41.20148340720281</v>
+        <v>47.46523039018463</v>
       </c>
     </row>
     <row r="288">
@@ -21475,13 +21475,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R288" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S288" t="n">
-        <v>40.03518773965074</v>
+        <v>46.26390905156617</v>
       </c>
       <c r="T288" t="n">
-        <v>40.03518773965074</v>
+        <v>46.26390905156617</v>
       </c>
     </row>
     <row r="289">
@@ -21549,13 +21549,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R289" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S289" t="n">
-        <v>39.25765729461603</v>
+        <v>45.46302815915386</v>
       </c>
       <c r="T289" t="n">
-        <v>39.25765729461603</v>
+        <v>45.46302815915386</v>
       </c>
     </row>
     <row r="290">
@@ -21623,13 +21623,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R290" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S290" t="n">
-        <v>38.86889207209867</v>
+        <v>45.06258771294771</v>
       </c>
       <c r="T290" t="n">
-        <v>38.86889207209867</v>
+        <v>45.06258771294771</v>
       </c>
     </row>
     <row r="291">
@@ -21697,13 +21697,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R291" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S291" t="n">
-        <v>38.71338598309173</v>
+        <v>44.90241153446525</v>
       </c>
       <c r="T291" t="n">
-        <v>38.71338598309173</v>
+        <v>44.90241153446525</v>
       </c>
     </row>
     <row r="292">
@@ -21771,13 +21771,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R292" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S292" t="n">
-        <v>38.63563293858826</v>
+        <v>44.82232344522401</v>
       </c>
       <c r="T292" t="n">
-        <v>38.63563293858826</v>
+        <v>44.82232344522401</v>
       </c>
     </row>
     <row r="293">
@@ -21845,13 +21845,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R293" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S293" t="n">
-        <v>35.52551115844942</v>
+        <v>41.61879987557479</v>
       </c>
       <c r="T293" t="n">
-        <v>35.52551115844942</v>
+        <v>41.61879987557479</v>
       </c>
     </row>
     <row r="294">
@@ -21919,13 +21919,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R294" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S294" t="n">
-        <v>29.30526759817174</v>
+        <v>35.21175273627635</v>
       </c>
       <c r="T294" t="n">
-        <v>29.30526759817174</v>
+        <v>35.21175273627635</v>
       </c>
     </row>
     <row r="295">
@@ -21995,13 +21995,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R295" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S295" t="n">
-        <v>43.48172003081821</v>
+        <v>49.81394606259898</v>
       </c>
       <c r="T295" t="n">
-        <v>43.48172003081821</v>
+        <v>49.81394606259898</v>
       </c>
     </row>
     <row r="296">
@@ -22069,13 +22069,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R296" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S296" t="n">
-        <v>41.55900861333959</v>
+        <v>47.83349263377811</v>
       </c>
       <c r="T296" t="n">
-        <v>41.55900861333959</v>
+        <v>47.83349263377811</v>
       </c>
     </row>
     <row r="297">
@@ -22143,13 +22143,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R297" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S297" t="n">
-        <v>40.40538176285243</v>
+        <v>46.64522057648561</v>
       </c>
       <c r="T297" t="n">
-        <v>40.40538176285243</v>
+        <v>46.64522057648561</v>
       </c>
     </row>
     <row r="298">
@@ -22217,13 +22217,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R298" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S298" t="n">
-        <v>40.32847330615328</v>
+        <v>46.56600243933277</v>
       </c>
       <c r="T298" t="n">
-        <v>40.32847330615328</v>
+        <v>46.56600243933277</v>
       </c>
     </row>
     <row r="299">
@@ -22291,13 +22291,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R299" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S299" t="n">
-        <v>36.48305047119606</v>
+        <v>42.60509558169105</v>
       </c>
       <c r="T299" t="n">
-        <v>36.48305047119606</v>
+        <v>42.60509558169105</v>
       </c>
     </row>
     <row r="300">
@@ -22365,13 +22365,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R300" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S300" t="n">
-        <v>33.791254486726</v>
+        <v>39.83246078134184</v>
       </c>
       <c r="T300" t="n">
-        <v>33.791254486726</v>
+        <v>39.83246078134184</v>
       </c>
     </row>
     <row r="301">
@@ -22439,13 +22439,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R301" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S301" t="n">
-        <v>33.63743757332772</v>
+        <v>39.67402450703618</v>
       </c>
       <c r="T301" t="n">
-        <v>33.63743757332772</v>
+        <v>39.67402450703618</v>
       </c>
     </row>
     <row r="302">
@@ -22513,13 +22513,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R302" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S302" t="n">
-        <v>31.33018387235338</v>
+        <v>37.29748039245115</v>
       </c>
       <c r="T302" t="n">
-        <v>31.33018387235338</v>
+        <v>37.29748039245115</v>
       </c>
     </row>
     <row r="303">
@@ -22587,13 +22587,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R303" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S303" t="n">
-        <v>30.17655702186621</v>
+        <v>36.10920833515863</v>
       </c>
       <c r="T303" t="n">
-        <v>30.17655702186621</v>
+        <v>36.10920833515863</v>
       </c>
     </row>
     <row r="304">
@@ -22661,13 +22661,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R304" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S304" t="n">
-        <v>30.09964856516707</v>
+        <v>36.02999019800579</v>
       </c>
       <c r="T304" t="n">
-        <v>30.09964856516707</v>
+        <v>36.02999019800579</v>
       </c>
     </row>
     <row r="305">
@@ -22735,13 +22735,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R305" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S305" t="n">
-        <v>29.71510628167135</v>
+        <v>35.63389951224163</v>
       </c>
       <c r="T305" t="n">
-        <v>29.71510628167135</v>
+        <v>35.63389951224163</v>
       </c>
     </row>
     <row r="306">
@@ -22809,13 +22809,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R306" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S306" t="n">
-        <v>18.94792234379112</v>
+        <v>24.54336031084481</v>
       </c>
       <c r="T306" t="n">
-        <v>18.94792234379112</v>
+        <v>24.54336031084481</v>
       </c>
     </row>
     <row r="307">
@@ -22883,13 +22883,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R307" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S307" t="n">
-        <v>17.0252109263125</v>
+        <v>22.56290688202395</v>
       </c>
       <c r="T307" t="n">
-        <v>17.0252109263125</v>
+        <v>22.56290688202395</v>
       </c>
     </row>
     <row r="308">
@@ -22957,13 +22957,13 @@
         <v>1.867959999999982</v>
       </c>
       <c r="R308" t="n">
-        <v>0</v>
+        <v>12.04644873936213</v>
       </c>
       <c r="S308" t="n">
-        <v>13.17978809135528</v>
+        <v>18.60200002438222</v>
       </c>
       <c r="T308" t="n">
-        <v>13.17978809135528</v>
+        <v>18.60200002438222</v>
       </c>
     </row>
     <row r="309">
@@ -23036,10 +23036,10 @@
         <v>0</v>
       </c>
       <c r="S309" t="n">
-        <v>77.77487693055934</v>
+        <v>76.85152652189421</v>
       </c>
       <c r="T309" t="n">
-        <v>77.77487693055934</v>
+        <v>76.85152652189421</v>
       </c>
     </row>
     <row r="310">
@@ -23110,10 +23110,10 @@
         <v>0</v>
       </c>
       <c r="S310" t="n">
-        <v>72.13239745504723</v>
+        <v>71.03959462054658</v>
       </c>
       <c r="T310" t="n">
-        <v>72.13239745504723</v>
+        <v>71.03959462054658</v>
       </c>
     </row>
     <row r="311">
@@ -23184,10 +23184,10 @@
         <v>0</v>
       </c>
       <c r="S311" t="n">
-        <v>69.92423151900158</v>
+        <v>68.76511403043187</v>
       </c>
       <c r="T311" t="n">
-        <v>69.92423151900158</v>
+        <v>68.76511403043187</v>
       </c>
     </row>
     <row r="312">
@@ -23258,10 +23258,10 @@
         <v>0</v>
       </c>
       <c r="S312" t="n">
-        <v>69.59811457466904</v>
+        <v>68.42920328754622</v>
       </c>
       <c r="T312" t="n">
-        <v>69.59811457466904</v>
+        <v>68.42920328754622</v>
       </c>
     </row>
     <row r="313">
@@ -23332,10 +23332,10 @@
         <v>0</v>
       </c>
       <c r="S313" t="n">
-        <v>62.40153680158996</v>
+        <v>61.01650110202493</v>
       </c>
       <c r="T313" t="n">
-        <v>62.40153680158996</v>
+        <v>61.01650110202493</v>
       </c>
     </row>
     <row r="314">
@@ -23406,10 +23406,10 @@
         <v>0</v>
       </c>
       <c r="S314" t="n">
-        <v>62.48352447512649</v>
+        <v>61.10095099278877</v>
       </c>
       <c r="T314" t="n">
-        <v>62.48352447512649</v>
+        <v>61.10095099278877</v>
       </c>
     </row>
     <row r="315">
@@ -23480,10 +23480,10 @@
         <v>0</v>
       </c>
       <c r="S315" t="n">
-        <v>63.38355513421478</v>
+        <v>62.02801097102137</v>
       </c>
       <c r="T315" t="n">
-        <v>63.38355513421478</v>
+        <v>62.02801097102137</v>
       </c>
     </row>
     <row r="316">
@@ -23554,10 +23554,10 @@
         <v>0</v>
       </c>
       <c r="S316" t="n">
-        <v>61.01233072600287</v>
+        <v>59.58557500946385</v>
       </c>
       <c r="T316" t="n">
-        <v>61.01233072600287</v>
+        <v>59.58557500946385</v>
       </c>
     </row>
     <row r="317">
@@ -23628,10 +23628,10 @@
         <v>0</v>
       </c>
       <c r="S317" t="n">
-        <v>61.50333989231527</v>
+        <v>60.09132994396207</v>
       </c>
       <c r="T317" t="n">
-        <v>61.50333989231527</v>
+        <v>60.09132994396207</v>
       </c>
     </row>
     <row r="318">
@@ -23702,10 +23702,10 @@
         <v>0</v>
       </c>
       <c r="S318" t="n">
-        <v>56.10590656250595</v>
+        <v>54.53180330482109</v>
       </c>
       <c r="T318" t="n">
-        <v>56.10590656250595</v>
+        <v>54.53180330482109</v>
       </c>
     </row>
     <row r="319">
@@ -23776,10 +23776,10 @@
         <v>0</v>
       </c>
       <c r="S319" t="n">
-        <v>54.14370364706991</v>
+        <v>52.51067238699794</v>
       </c>
       <c r="T319" t="n">
-        <v>54.14370364706991</v>
+        <v>52.51067238699794</v>
       </c>
     </row>
     <row r="320">
@@ -23850,10 +23850,10 @@
         <v>0</v>
       </c>
       <c r="S320" t="n">
-        <v>60.63738792751113</v>
+        <v>59.19937209615384</v>
       </c>
       <c r="T320" t="n">
-        <v>60.63738792751113</v>
+        <v>59.19937209615384</v>
       </c>
     </row>
     <row r="321">
@@ -23924,10 +23924,10 @@
         <v>0</v>
       </c>
       <c r="S321" t="n">
-        <v>54.55272513984579</v>
+        <v>52.93197743073232</v>
       </c>
       <c r="T321" t="n">
-        <v>54.55272513984579</v>
+        <v>52.93197743073232</v>
       </c>
     </row>
     <row r="322">
@@ -23998,10 +23998,10 @@
         <v>0</v>
       </c>
       <c r="S322" t="n">
-        <v>54.22660819551325</v>
+        <v>52.59606668784667</v>
       </c>
       <c r="T322" t="n">
-        <v>54.22660819551325</v>
+        <v>52.59606668784667</v>
       </c>
     </row>
     <row r="323">
@@ -24072,10 +24072,10 @@
         <v>0</v>
       </c>
       <c r="S323" t="n">
-        <v>58.88890308821417</v>
+        <v>57.39837754036764</v>
       </c>
       <c r="T323" t="n">
-        <v>58.88890308821417</v>
+        <v>57.39837754036764</v>
       </c>
     </row>
     <row r="324">
@@ -24215,13 +24215,13 @@
         <v>-0.3366600000000091</v>
       </c>
       <c r="R325" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S325" t="n">
-        <v>48.02713322646</v>
+        <v>55.15171017832049</v>
       </c>
       <c r="T325" t="n">
-        <v>48.02713322646</v>
+        <v>55.15171017832049</v>
       </c>
     </row>
     <row r="326">
@@ -24289,13 +24289,13 @@
         <v>-0.3366600000000091</v>
       </c>
       <c r="R326" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S326" t="n">
-        <v>47.84805215114729</v>
+        <v>54.9672510200631</v>
       </c>
       <c r="T326" t="n">
-        <v>47.84805215114729</v>
+        <v>54.9672510200631</v>
       </c>
     </row>
     <row r="327">
@@ -24363,13 +24363,13 @@
         <v>-3.643590000000017</v>
       </c>
       <c r="R327" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S327" t="n">
-        <v>45.46080513978893</v>
+        <v>52.508311271691</v>
       </c>
       <c r="T327" t="n">
-        <v>45.46080513978893</v>
+        <v>52.508311271691</v>
       </c>
     </row>
     <row r="328">
@@ -24437,13 +24437,13 @@
         <v>-3.643590000000017</v>
       </c>
       <c r="R328" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S328" t="n">
-        <v>45.19218352681987</v>
+        <v>52.23162253430491</v>
       </c>
       <c r="T328" t="n">
-        <v>45.19218352681987</v>
+        <v>52.23162253430491</v>
       </c>
     </row>
     <row r="329">
@@ -24511,13 +24511,13 @@
         <v>-0.3366600000000091</v>
       </c>
       <c r="R329" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S329" t="n">
-        <v>47.13172784989645</v>
+        <v>54.22941438703353</v>
       </c>
       <c r="T329" t="n">
-        <v>47.13172784989645</v>
+        <v>54.22941438703353</v>
       </c>
     </row>
     <row r="330">
@@ -24585,13 +24585,13 @@
         <v>-0.3366600000000091</v>
       </c>
       <c r="R330" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S330" t="n">
-        <v>46.68402516161468</v>
+        <v>53.76826649139005</v>
       </c>
       <c r="T330" t="n">
-        <v>46.68402516161468</v>
+        <v>53.76826649139005</v>
       </c>
     </row>
     <row r="331">
@@ -24659,13 +24659,13 @@
         <v>-3.643590000000017</v>
       </c>
       <c r="R331" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S331" t="n">
-        <v>39.10342696618775</v>
+        <v>45.96001115355359</v>
       </c>
       <c r="T331" t="n">
-        <v>39.10342696618775</v>
+        <v>45.96001115355359</v>
       </c>
     </row>
     <row r="332">
@@ -24733,13 +24733,13 @@
         <v>-3.643590000000017</v>
       </c>
       <c r="R332" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S332" t="n">
-        <v>36.41721083649712</v>
+        <v>43.19312377969272</v>
       </c>
       <c r="T332" t="n">
-        <v>36.41721083649712</v>
+        <v>43.19312377969272</v>
       </c>
     </row>
     <row r="333">
@@ -24807,7 +24807,7 @@
         <v>-0.3366600000000091</v>
       </c>
       <c r="R333" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S333" t="inlineStr"/>
       <c r="T333" t="inlineStr"/>
@@ -24882,10 +24882,10 @@
         <v>0</v>
       </c>
       <c r="S334" t="n">
-        <v>69.91391360400101</v>
+        <v>68.75448625241202</v>
       </c>
       <c r="T334" t="n">
-        <v>69.91391360400101</v>
+        <v>68.75448625241202</v>
       </c>
     </row>
     <row r="335">
@@ -24956,10 +24956,10 @@
         <v>0</v>
       </c>
       <c r="S335" t="n">
-        <v>69.11373296381183</v>
+        <v>67.93027494429131</v>
       </c>
       <c r="T335" t="n">
-        <v>69.11373296381183</v>
+        <v>67.93027494429131</v>
       </c>
     </row>
     <row r="336">
@@ -25030,10 +25030,10 @@
         <v>0</v>
       </c>
       <c r="S336" t="n">
-        <v>67.91346200352808</v>
+        <v>66.69395798211019</v>
       </c>
       <c r="T336" t="n">
-        <v>67.91346200352808</v>
+        <v>66.69395798211019</v>
       </c>
     </row>
     <row r="337">
@@ -25104,10 +25104,10 @@
         <v>0</v>
       </c>
       <c r="S337" t="n">
-        <v>67.75342587549025</v>
+        <v>66.52911572048606</v>
       </c>
       <c r="T337" t="n">
-        <v>67.75342587549025</v>
+        <v>66.52911572048606</v>
       </c>
     </row>
     <row r="338">
@@ -25178,10 +25178,10 @@
         <v>0</v>
       </c>
       <c r="S338" t="n">
-        <v>67.35333555539566</v>
+        <v>66.11701006642568</v>
       </c>
       <c r="T338" t="n">
-        <v>67.35333555539566</v>
+        <v>66.11701006642568</v>
       </c>
     </row>
     <row r="339">
@@ -25252,10 +25252,10 @@
         <v>0</v>
       </c>
       <c r="S339" t="n">
-        <v>65.75297427501732</v>
+        <v>64.46858745018423</v>
       </c>
       <c r="T339" t="n">
-        <v>65.75297427501732</v>
+        <v>64.46858745018423</v>
       </c>
     </row>
     <row r="340">
@@ -25326,10 +25326,10 @@
         <v>0</v>
       </c>
       <c r="S340" t="n">
-        <v>60.9518904338823</v>
+        <v>59.52331960145984</v>
       </c>
       <c r="T340" t="n">
-        <v>60.9518904338823</v>
+        <v>59.52331960145984</v>
       </c>
     </row>
     <row r="341">
@@ -25400,10 +25400,10 @@
         <v>0</v>
       </c>
       <c r="S341" t="n">
-        <v>54.7428212968908</v>
+        <v>53.12778247074147</v>
       </c>
       <c r="T341" t="n">
-        <v>54.7428212968908</v>
+        <v>53.12778247074147</v>
       </c>
     </row>
     <row r="342">
@@ -25474,10 +25474,10 @@
         <v>0</v>
       </c>
       <c r="S342" t="n">
-        <v>51.34972275161226</v>
+        <v>49.63278390401106</v>
       </c>
       <c r="T342" t="n">
-        <v>51.34972275161226</v>
+        <v>49.63278390401106</v>
       </c>
     </row>
     <row r="343">
@@ -25548,10 +25548,10 @@
         <v>0</v>
       </c>
       <c r="S343" t="n">
-        <v>50.3736132475403</v>
+        <v>48.62736031486994</v>
       </c>
       <c r="T343" t="n">
-        <v>50.3736132475403</v>
+        <v>48.62736031486994</v>
       </c>
     </row>
     <row r="344">
@@ -25624,10 +25624,10 @@
         <v>0</v>
       </c>
       <c r="S344" t="n">
-        <v>70.56091784655945</v>
+        <v>69.42092103767837</v>
       </c>
       <c r="T344" t="n">
-        <v>70.56091784655945</v>
+        <v>69.42092103767837</v>
       </c>
     </row>
     <row r="345">
@@ -25698,10 +25698,10 @@
         <v>0</v>
       </c>
       <c r="S345" t="n">
-        <v>73.45573829576384</v>
+        <v>72.40267744289375</v>
       </c>
       <c r="T345" t="n">
-        <v>73.45573829576384</v>
+        <v>72.40267744289375</v>
       </c>
     </row>
     <row r="346">
@@ -25772,10 +25772,10 @@
         <v>0</v>
       </c>
       <c r="S346" t="n">
-        <v>67.9526125501819</v>
+        <v>66.73428428051145</v>
       </c>
       <c r="T346" t="n">
-        <v>67.9526125501819</v>
+        <v>66.73428428051145</v>
       </c>
     </row>
     <row r="347">
@@ -25846,10 +25846,10 @@
         <v>0</v>
       </c>
       <c r="S347" t="n">
-        <v>69.07398461273689</v>
+        <v>67.88933288847329</v>
       </c>
       <c r="T347" t="n">
-        <v>69.07398461273689</v>
+        <v>67.88933288847329</v>
       </c>
     </row>
     <row r="348">
@@ -25920,10 +25920,10 @@
         <v>0</v>
       </c>
       <c r="S348" t="n">
-        <v>64.69223092970995</v>
+        <v>63.37598833405283</v>
       </c>
       <c r="T348" t="n">
-        <v>64.69223092970995</v>
+        <v>63.37598833405283</v>
       </c>
     </row>
     <row r="349">
@@ -25994,10 +25994,10 @@
         <v>0</v>
       </c>
       <c r="S349" t="n">
-        <v>64.42547135615536</v>
+        <v>63.10121755601802</v>
       </c>
       <c r="T349" t="n">
-        <v>64.42547135615536</v>
+        <v>63.10121755601802</v>
       </c>
     </row>
     <row r="350">
@@ -26068,10 +26068,10 @@
         <v>0</v>
       </c>
       <c r="S350" t="n">
-        <v>61.38244851038155</v>
+        <v>59.96680800598997</v>
       </c>
       <c r="T350" t="n">
-        <v>61.38244851038155</v>
+        <v>59.96680800598997</v>
       </c>
     </row>
     <row r="351">
@@ -26142,10 +26142,10 @@
         <v>0</v>
       </c>
       <c r="S351" t="n">
-        <v>58.30484747554338</v>
+        <v>56.79678183015296</v>
       </c>
       <c r="T351" t="n">
-        <v>58.30484747554338</v>
+        <v>56.79678183015296</v>
       </c>
     </row>
     <row r="352">
@@ -26216,10 +26216,10 @@
         <v>0</v>
       </c>
       <c r="S352" t="n">
-        <v>56.16583791762645</v>
+        <v>54.59353449165615</v>
       </c>
       <c r="T352" t="n">
-        <v>56.16583791762645</v>
+        <v>54.59353449165615</v>
       </c>
     </row>
     <row r="353">
@@ -26292,10 +26292,10 @@
         <v>0</v>
       </c>
       <c r="S353" t="n">
-        <v>60.33865245590198</v>
+        <v>58.89166513416232</v>
       </c>
       <c r="T353" t="n">
-        <v>60.33865245590198</v>
+        <v>58.89166513416232</v>
       </c>
     </row>
     <row r="354">
@@ -26366,10 +26366,10 @@
         <v>0</v>
       </c>
       <c r="S354" t="n">
-        <v>65.2987149093033</v>
+        <v>64.00068596989755</v>
       </c>
       <c r="T354" t="n">
-        <v>65.2987149093033</v>
+        <v>64.00068596989755</v>
       </c>
     </row>
     <row r="355">
@@ -26440,10 +26440,10 @@
         <v>0</v>
       </c>
       <c r="S355" t="n">
-        <v>61.35724741886809</v>
+        <v>59.94085008654134</v>
       </c>
       <c r="T355" t="n">
-        <v>61.35724741886809</v>
+        <v>59.94085008654134</v>
       </c>
     </row>
     <row r="356">
@@ -26514,10 +26514,10 @@
         <v>0</v>
       </c>
       <c r="S356" t="n">
-        <v>61.96508624374651</v>
+        <v>60.56694325578018</v>
       </c>
       <c r="T356" t="n">
-        <v>61.96508624374651</v>
+        <v>60.56694325578018</v>
       </c>
     </row>
     <row r="357">
@@ -26588,10 +26588,10 @@
         <v>0</v>
       </c>
       <c r="S357" t="n">
-        <v>58.56972831266407</v>
+        <v>57.06961745037959</v>
       </c>
       <c r="T357" t="n">
-        <v>58.56972831266407</v>
+        <v>57.06961745037959</v>
       </c>
     </row>
     <row r="358">
@@ -26662,10 +26662,10 @@
         <v>0</v>
       </c>
       <c r="S358" t="n">
-        <v>55.30496584676121</v>
+        <v>53.70680909489487</v>
       </c>
       <c r="T358" t="n">
-        <v>55.30496584676121</v>
+        <v>53.70680909489487</v>
       </c>
     </row>
     <row r="359">
@@ -26736,10 +26736,10 @@
         <v>0</v>
       </c>
       <c r="S359" t="n">
-        <v>57.3825363176273</v>
+        <v>55.84677223509371</v>
       </c>
       <c r="T359" t="n">
-        <v>57.3825363176273</v>
+        <v>55.84677223509371</v>
       </c>
     </row>
     <row r="360">
@@ -26810,10 +26810,10 @@
         <v>0</v>
       </c>
       <c r="S360" t="n">
-        <v>61.47832697187659</v>
+        <v>60.06556584665797</v>
       </c>
       <c r="T360" t="n">
-        <v>61.47832697187659</v>
+        <v>60.06556584665797</v>
       </c>
     </row>
     <row r="361">
@@ -26884,10 +26884,10 @@
         <v>0</v>
       </c>
       <c r="S361" t="n">
-        <v>48.79916861359001</v>
+        <v>47.00563266221759</v>
       </c>
       <c r="T361" t="n">
-        <v>48.79916861359001</v>
+        <v>47.00563266221759</v>
       </c>
     </row>
     <row r="362">
@@ -26958,10 +26958,10 @@
         <v>0</v>
       </c>
       <c r="S362" t="n">
-        <v>54.52139305568383</v>
+        <v>52.89970439539973</v>
       </c>
       <c r="T362" t="n">
-        <v>54.52139305568383</v>
+        <v>52.89970439539973</v>
       </c>
     </row>
     <row r="363">
@@ -27032,10 +27032,10 @@
         <v>0</v>
       </c>
       <c r="S363" t="n">
-        <v>44.59651019279568</v>
+        <v>42.67676187902967</v>
       </c>
       <c r="T363" t="n">
-        <v>44.59651019279568</v>
+        <v>42.67676187902967</v>
       </c>
     </row>
     <row r="364">
@@ -27106,10 +27106,10 @@
         <v>0</v>
       </c>
       <c r="S364" t="n">
-        <v>40.93996133135411</v>
+        <v>38.91040117379737</v>
       </c>
       <c r="T364" t="n">
-        <v>40.93996133135411</v>
+        <v>38.91040117379737</v>
       </c>
     </row>
     <row r="365">
@@ -27252,10 +27252,10 @@
         <v>0</v>
       </c>
       <c r="S366" t="n">
-        <v>63.41272973293118</v>
+        <v>62.05806172826819</v>
       </c>
       <c r="T366" t="n">
-        <v>63.41272973293118</v>
+        <v>62.05806172826819</v>
       </c>
     </row>
     <row r="367">
@@ -27326,10 +27326,10 @@
         <v>0</v>
       </c>
       <c r="S367" t="n">
-        <v>61.97709414952537</v>
+        <v>60.57931177762726</v>
       </c>
       <c r="T367" t="n">
-        <v>61.97709414952537</v>
+        <v>60.57931177762726</v>
       </c>
     </row>
     <row r="368">
@@ -27400,10 +27400,10 @@
         <v>0</v>
       </c>
       <c r="S368" t="n">
-        <v>63.91379872364339</v>
+        <v>62.57417859932374</v>
       </c>
       <c r="T368" t="n">
-        <v>63.91379872364339</v>
+        <v>62.57417859932374</v>
       </c>
     </row>
     <row r="369">
@@ -27474,10 +27474,10 @@
         <v>0</v>
       </c>
       <c r="S369" t="n">
-        <v>60.3483259779596</v>
+        <v>58.90162916711789</v>
       </c>
       <c r="T369" t="n">
-        <v>60.3483259779596</v>
+        <v>58.90162916711789</v>
       </c>
     </row>
     <row r="370">
@@ -27548,10 +27548,10 @@
         <v>0</v>
       </c>
       <c r="S370" t="n">
-        <v>60.23974143318856</v>
+        <v>58.7897836597506</v>
       </c>
       <c r="T370" t="n">
-        <v>60.23974143318856</v>
+        <v>58.7897836597506</v>
       </c>
     </row>
     <row r="371">
@@ -27622,10 +27622,10 @@
         <v>0</v>
       </c>
       <c r="S371" t="n">
-        <v>54.03798384199615</v>
+        <v>52.40177765191223</v>
       </c>
       <c r="T371" t="n">
-        <v>54.03798384199615</v>
+        <v>52.40177765191223</v>
       </c>
     </row>
     <row r="372">
@@ -27696,10 +27696,10 @@
         <v>0</v>
       </c>
       <c r="S372" t="n">
-        <v>55.08197555656363</v>
+        <v>53.47712205980423</v>
       </c>
       <c r="T372" t="n">
-        <v>55.08197555656363</v>
+        <v>53.47712205980423</v>
       </c>
     </row>
     <row r="373">
@@ -27770,10 +27770,10 @@
         <v>0</v>
       </c>
       <c r="S373" t="n">
-        <v>53.33840357060556</v>
+        <v>51.68118789797619</v>
       </c>
       <c r="T373" t="n">
-        <v>53.33840357060556</v>
+        <v>51.68118789797619</v>
       </c>
     </row>
     <row r="374">
@@ -27844,10 +27844,10 @@
         <v>0</v>
       </c>
       <c r="S374" t="n">
-        <v>46.82333088434249</v>
+        <v>44.97045745593867</v>
       </c>
       <c r="T374" t="n">
-        <v>46.82333088434249</v>
+        <v>44.97045745593867</v>
       </c>
     </row>
     <row r="375">
@@ -27918,10 +27918,10 @@
         <v>0</v>
       </c>
       <c r="S375" t="n">
-        <v>43.40913699367562</v>
+        <v>41.45373001782033</v>
       </c>
       <c r="T375" t="n">
-        <v>43.40913699367562</v>
+        <v>41.45373001782033</v>
       </c>
     </row>
   </sheetData>

</xml_diff>